<commit_message>
Add random forest experiments and model evaluation analysis
</commit_message>
<xml_diff>
--- a/results/random_forest/all_predictions.xlsx
+++ b/results/random_forest/all_predictions.xlsx
@@ -1146,16 +1146,16 @@
         <v>147000</v>
       </c>
       <c r="CC2" t="n">
-        <v>127104.74</v>
+        <v>126136.6261727305</v>
       </c>
       <c r="CD2" t="n">
-        <v>19895.25999999999</v>
+        <v>20863.37382726952</v>
       </c>
       <c r="CE2" t="n">
-        <v>19895.25999999999</v>
+        <v>20863.37382726952</v>
       </c>
       <c r="CF2" t="n">
-        <v>13.53419047619047</v>
+        <v>14.1927713110677</v>
       </c>
     </row>
     <row r="3">
@@ -1466,16 +1466,16 @@
         <v>132500</v>
       </c>
       <c r="CC3" t="n">
-        <v>138627.85</v>
+        <v>140129.4504584503</v>
       </c>
       <c r="CD3" t="n">
-        <v>-6127.850000000006</v>
+        <v>-7629.45045845033</v>
       </c>
       <c r="CE3" t="n">
-        <v>6127.850000000006</v>
+        <v>7629.45045845033</v>
       </c>
       <c r="CF3" t="n">
-        <v>4.624792452830193</v>
+        <v>5.758075817698362</v>
       </c>
     </row>
     <row r="4">
@@ -1790,16 +1790,16 @@
         <v>305000</v>
       </c>
       <c r="CC4" t="n">
-        <v>302258.49</v>
+        <v>301900.6418884548</v>
       </c>
       <c r="CD4" t="n">
-        <v>2741.510000000009</v>
+        <v>3099.358111545152</v>
       </c>
       <c r="CE4" t="n">
-        <v>2741.510000000009</v>
+        <v>3099.358111545152</v>
       </c>
       <c r="CF4" t="n">
-        <v>0.8988557377049211</v>
+        <v>1.016182987391853</v>
       </c>
     </row>
     <row r="5">
@@ -2114,16 +2114,16 @@
         <v>335000</v>
       </c>
       <c r="CC5" t="n">
-        <v>356133.38</v>
+        <v>350636.7986870643</v>
       </c>
       <c r="CD5" t="n">
-        <v>-21133.38</v>
+        <v>-15636.79868706432</v>
       </c>
       <c r="CE5" t="n">
-        <v>21133.38</v>
+        <v>15636.79868706432</v>
       </c>
       <c r="CF5" t="n">
-        <v>6.308471641791045</v>
+        <v>4.667701100616215</v>
       </c>
     </row>
     <row r="6">
@@ -2434,16 +2434,16 @@
         <v>153500</v>
       </c>
       <c r="CC6" t="n">
-        <v>170540.05</v>
+        <v>169382.3071196936</v>
       </c>
       <c r="CD6" t="n">
-        <v>-17040.04999999999</v>
+        <v>-15882.30711969361</v>
       </c>
       <c r="CE6" t="n">
-        <v>17040.04999999999</v>
+        <v>15882.30711969361</v>
       </c>
       <c r="CF6" t="n">
-        <v>11.10100977198696</v>
+        <v>10.34677988253655</v>
       </c>
     </row>
     <row r="7">
@@ -2758,16 +2758,16 @@
         <v>239000</v>
       </c>
       <c r="CC7" t="n">
-        <v>201788.5</v>
+        <v>203669.6846245257</v>
       </c>
       <c r="CD7" t="n">
-        <v>37211.5</v>
+        <v>35330.31537547431</v>
       </c>
       <c r="CE7" t="n">
-        <v>37211.5</v>
+        <v>35330.31537547431</v>
       </c>
       <c r="CF7" t="n">
-        <v>15.56966527196653</v>
+        <v>14.78255873450808</v>
       </c>
     </row>
     <row r="8">
@@ -3080,16 +3080,16 @@
         <v>200000</v>
       </c>
       <c r="CC8" t="n">
-        <v>208194.14</v>
+        <v>206975.5376792615</v>
       </c>
       <c r="CD8" t="n">
-        <v>-8194.140000000014</v>
+        <v>-6975.537679261528</v>
       </c>
       <c r="CE8" t="n">
-        <v>8194.140000000014</v>
+        <v>6975.537679261528</v>
       </c>
       <c r="CF8" t="n">
-        <v>4.097070000000007</v>
+        <v>3.487768839630764</v>
       </c>
     </row>
     <row r="9">
@@ -3402,16 +3402,16 @@
         <v>165000</v>
       </c>
       <c r="CC9" t="n">
-        <v>163618.32</v>
+        <v>164646.5931569762</v>
       </c>
       <c r="CD9" t="n">
-        <v>1381.679999999993</v>
+        <v>353.406843023753</v>
       </c>
       <c r="CE9" t="n">
-        <v>1381.679999999993</v>
+        <v>353.406843023753</v>
       </c>
       <c r="CF9" t="n">
-        <v>0.837381818181814</v>
+        <v>0.2141859654689412</v>
       </c>
     </row>
     <row r="10">
@@ -3722,16 +3722,16 @@
         <v>100000</v>
       </c>
       <c r="CC10" t="n">
-        <v>118704.52</v>
+        <v>119435.8510420022</v>
       </c>
       <c r="CD10" t="n">
-        <v>-18704.52</v>
+        <v>-19435.85104200216</v>
       </c>
       <c r="CE10" t="n">
-        <v>18704.52</v>
+        <v>19435.85104200216</v>
       </c>
       <c r="CF10" t="n">
-        <v>18.70452000000001</v>
+        <v>19.43585104200216</v>
       </c>
     </row>
     <row r="11">
@@ -4044,16 +4044,16 @@
         <v>277000</v>
       </c>
       <c r="CC11" t="n">
-        <v>245907.6</v>
+        <v>248887.7847611712</v>
       </c>
       <c r="CD11" t="n">
-        <v>31092.39999999999</v>
+        <v>28112.21523882879</v>
       </c>
       <c r="CE11" t="n">
-        <v>31092.39999999999</v>
+        <v>28112.21523882879</v>
       </c>
       <c r="CF11" t="n">
-        <v>11.22469314079422</v>
+        <v>10.14881416564216</v>
       </c>
     </row>
     <row r="12">
@@ -4366,16 +4366,16 @@
         <v>137000</v>
       </c>
       <c r="CC12" t="n">
-        <v>130915</v>
+        <v>129124.2390255876</v>
       </c>
       <c r="CD12" t="n">
-        <v>6085</v>
+        <v>7875.760974412391</v>
       </c>
       <c r="CE12" t="n">
-        <v>6085</v>
+        <v>7875.760974412391</v>
       </c>
       <c r="CF12" t="n">
-        <v>4.441605839416058</v>
+        <v>5.74873063825722</v>
       </c>
     </row>
     <row r="13">
@@ -4690,16 +4690,16 @@
         <v>250000</v>
       </c>
       <c r="CC13" t="n">
-        <v>222620.85</v>
+        <v>224170.5604246765</v>
       </c>
       <c r="CD13" t="n">
-        <v>27379.14999999999</v>
+        <v>25829.43957532349</v>
       </c>
       <c r="CE13" t="n">
-        <v>27379.14999999999</v>
+        <v>25829.43957532349</v>
       </c>
       <c r="CF13" t="n">
-        <v>10.95166</v>
+        <v>10.33177583012939</v>
       </c>
     </row>
     <row r="14">
@@ -5010,16 +5010,16 @@
         <v>126500</v>
       </c>
       <c r="CC14" t="n">
-        <v>134084.5</v>
+        <v>136059.3466097887</v>
       </c>
       <c r="CD14" t="n">
-        <v>-7584.5</v>
+        <v>-9559.346609788656</v>
       </c>
       <c r="CE14" t="n">
-        <v>7584.5</v>
+        <v>9559.346609788656</v>
       </c>
       <c r="CF14" t="n">
-        <v>5.995652173913044</v>
+        <v>7.556795738963364</v>
       </c>
     </row>
     <row r="15">
@@ -5338,16 +5338,16 @@
         <v>119900</v>
       </c>
       <c r="CC15" t="n">
-        <v>120364.5</v>
+        <v>121904.935615086</v>
       </c>
       <c r="CD15" t="n">
-        <v>-464.5</v>
+        <v>-2004.935615085997</v>
       </c>
       <c r="CE15" t="n">
-        <v>464.5</v>
+        <v>2004.935615085997</v>
       </c>
       <c r="CF15" t="n">
-        <v>0.3874061718098415</v>
+        <v>1.672173156869055</v>
       </c>
     </row>
     <row r="16">
@@ -5658,16 +5658,16 @@
         <v>66500</v>
       </c>
       <c r="CC16" t="n">
-        <v>104307.5</v>
+        <v>105664.4147162552</v>
       </c>
       <c r="CD16" t="n">
-        <v>-37807.5</v>
+        <v>-39164.41471625521</v>
       </c>
       <c r="CE16" t="n">
-        <v>37807.5</v>
+        <v>39164.41471625521</v>
       </c>
       <c r="CF16" t="n">
-        <v>56.85338345864661</v>
+        <v>58.89385671617325</v>
       </c>
     </row>
     <row r="17">
@@ -5976,16 +5976,16 @@
         <v>173000</v>
       </c>
       <c r="CC17" t="n">
-        <v>167311.82</v>
+        <v>167652.3792251153</v>
       </c>
       <c r="CD17" t="n">
-        <v>5688.179999999993</v>
+        <v>5347.620774884708</v>
       </c>
       <c r="CE17" t="n">
-        <v>5688.179999999993</v>
+        <v>5347.620774884708</v>
       </c>
       <c r="CF17" t="n">
-        <v>3.287965317919071</v>
+        <v>3.091110274499831</v>
       </c>
     </row>
     <row r="18">
@@ -6300,16 +6300,16 @@
         <v>266000</v>
       </c>
       <c r="CC18" t="n">
-        <v>253453.92</v>
+        <v>254065.0603356626</v>
       </c>
       <c r="CD18" t="n">
-        <v>12546.07999999999</v>
+        <v>11934.93966433738</v>
       </c>
       <c r="CE18" t="n">
-        <v>12546.07999999999</v>
+        <v>11934.93966433738</v>
       </c>
       <c r="CF18" t="n">
-        <v>4.716571428571424</v>
+        <v>4.486819422683224</v>
       </c>
     </row>
     <row r="19">
@@ -6630,16 +6630,16 @@
         <v>139900</v>
       </c>
       <c r="CC19" t="n">
-        <v>140402.24</v>
+        <v>139307.0830380256</v>
       </c>
       <c r="CD19" t="n">
-        <v>-502.2399999999907</v>
+        <v>592.916961974377</v>
       </c>
       <c r="CE19" t="n">
-        <v>502.2399999999907</v>
+        <v>592.916961974377</v>
       </c>
       <c r="CF19" t="n">
-        <v>0.3589992852037103</v>
+        <v>0.4238148405821137</v>
       </c>
     </row>
     <row r="20">
@@ -6930,16 +6930,16 @@
         <v>126000</v>
       </c>
       <c r="CC20" t="n">
-        <v>140503.47</v>
+        <v>142436.2443120942</v>
       </c>
       <c r="CD20" t="n">
-        <v>-14503.47</v>
+        <v>-16436.24431209423</v>
       </c>
       <c r="CE20" t="n">
-        <v>14503.47</v>
+        <v>16436.24431209423</v>
       </c>
       <c r="CF20" t="n">
-        <v>11.51069047619048</v>
+        <v>13.04463834293193</v>
       </c>
     </row>
     <row r="21">
@@ -7254,16 +7254,16 @@
         <v>129900</v>
       </c>
       <c r="CC21" t="n">
-        <v>141557</v>
+        <v>142353.3100518094</v>
       </c>
       <c r="CD21" t="n">
-        <v>-11657</v>
+        <v>-12453.31005180939</v>
       </c>
       <c r="CE21" t="n">
-        <v>11657</v>
+        <v>12453.31005180939</v>
       </c>
       <c r="CF21" t="n">
-        <v>8.973826020015396</v>
+        <v>9.586843765827087</v>
       </c>
     </row>
     <row r="22">
@@ -7578,16 +7578,16 @@
         <v>157900</v>
       </c>
       <c r="CC22" t="n">
-        <v>153131</v>
+        <v>153086.0676668057</v>
       </c>
       <c r="CD22" t="n">
-        <v>4769</v>
+        <v>4813.932333194301</v>
       </c>
       <c r="CE22" t="n">
-        <v>4769</v>
+        <v>4813.932333194301</v>
       </c>
       <c r="CF22" t="n">
-        <v>3.020265991133629</v>
+        <v>3.04872218695016</v>
       </c>
     </row>
     <row r="23">
@@ -7902,16 +7902,16 @@
         <v>185000</v>
       </c>
       <c r="CC23" t="n">
-        <v>183826</v>
+        <v>184104.7697970901</v>
       </c>
       <c r="CD23" t="n">
-        <v>1174</v>
+        <v>895.2302029099083</v>
       </c>
       <c r="CE23" t="n">
-        <v>1174</v>
+        <v>895.2302029099083</v>
       </c>
       <c r="CF23" t="n">
-        <v>0.6345945945945947</v>
+        <v>0.4839082177891396</v>
       </c>
     </row>
     <row r="24">
@@ -8222,16 +8222,16 @@
         <v>230000</v>
       </c>
       <c r="CC24" t="n">
-        <v>224265.27</v>
+        <v>222489.3363391258</v>
       </c>
       <c r="CD24" t="n">
-        <v>5734.73000000001</v>
+        <v>7510.663660874241</v>
       </c>
       <c r="CE24" t="n">
-        <v>5734.73000000001</v>
+        <v>7510.663660874241</v>
       </c>
       <c r="CF24" t="n">
-        <v>2.493360869565222</v>
+        <v>3.265505939510539</v>
       </c>
     </row>
     <row r="25">
@@ -8548,16 +8548,16 @@
         <v>165000</v>
       </c>
       <c r="CC25" t="n">
-        <v>147919.25</v>
+        <v>153089.011941824</v>
       </c>
       <c r="CD25" t="n">
-        <v>17080.75</v>
+        <v>11910.98805817601</v>
       </c>
       <c r="CE25" t="n">
-        <v>17080.75</v>
+        <v>11910.98805817601</v>
       </c>
       <c r="CF25" t="n">
-        <v>10.3519696969697</v>
+        <v>7.218780641318792</v>
       </c>
     </row>
     <row r="26">
@@ -8876,16 +8876,16 @@
         <v>135000</v>
       </c>
       <c r="CC26" t="n">
-        <v>138978.32</v>
+        <v>139716.3498070844</v>
       </c>
       <c r="CD26" t="n">
-        <v>-3978.320000000007</v>
+        <v>-4716.349807084363</v>
       </c>
       <c r="CE26" t="n">
-        <v>3978.320000000007</v>
+        <v>4716.349807084363</v>
       </c>
       <c r="CF26" t="n">
-        <v>2.946903703703709</v>
+        <v>3.493592449692121</v>
       </c>
     </row>
     <row r="27">
@@ -9200,16 +9200,16 @@
         <v>165000</v>
       </c>
       <c r="CC27" t="n">
-        <v>159488.75</v>
+        <v>159444.1629899106</v>
       </c>
       <c r="CD27" t="n">
-        <v>5511.25</v>
+        <v>5555.837010089395</v>
       </c>
       <c r="CE27" t="n">
-        <v>5511.25</v>
+        <v>5555.837010089395</v>
       </c>
       <c r="CF27" t="n">
-        <v>3.340151515151515</v>
+        <v>3.367173945508724</v>
       </c>
     </row>
     <row r="28">
@@ -9524,16 +9524,16 @@
         <v>184000</v>
       </c>
       <c r="CC28" t="n">
-        <v>194775</v>
+        <v>196727.8490879224</v>
       </c>
       <c r="CD28" t="n">
-        <v>-10775</v>
+        <v>-12727.8490879224</v>
       </c>
       <c r="CE28" t="n">
-        <v>10775</v>
+        <v>12727.8490879224</v>
       </c>
       <c r="CF28" t="n">
-        <v>5.855978260869565</v>
+        <v>6.917309286914346</v>
       </c>
     </row>
     <row r="29">
@@ -9848,16 +9848,16 @@
         <v>127500</v>
       </c>
       <c r="CC29" t="n">
-        <v>144500.52</v>
+        <v>143985.1850725465</v>
       </c>
       <c r="CD29" t="n">
-        <v>-17000.51999999999</v>
+        <v>-16485.18507254648</v>
       </c>
       <c r="CE29" t="n">
-        <v>17000.51999999999</v>
+        <v>16485.18507254648</v>
       </c>
       <c r="CF29" t="n">
-        <v>13.33374117647058</v>
+        <v>12.92955691964429</v>
       </c>
     </row>
     <row r="30">
@@ -10172,16 +10172,16 @@
         <v>159500</v>
       </c>
       <c r="CC30" t="n">
-        <v>166367.27</v>
+        <v>166449.2448433172</v>
       </c>
       <c r="CD30" t="n">
-        <v>-6867.26999999999</v>
+        <v>-6949.244843317167</v>
       </c>
       <c r="CE30" t="n">
-        <v>6867.26999999999</v>
+        <v>6949.244843317167</v>
       </c>
       <c r="CF30" t="n">
-        <v>4.305498432601874</v>
+        <v>4.356893318694149</v>
       </c>
     </row>
     <row r="31">
@@ -10500,16 +10500,16 @@
         <v>162900</v>
       </c>
       <c r="CC31" t="n">
-        <v>184801.5</v>
+        <v>185422.1908960568</v>
       </c>
       <c r="CD31" t="n">
-        <v>-21901.5</v>
+        <v>-22522.19089605683</v>
       </c>
       <c r="CE31" t="n">
-        <v>21901.5</v>
+        <v>22522.19089605683</v>
       </c>
       <c r="CF31" t="n">
-        <v>13.44475138121547</v>
+        <v>13.82577710009627</v>
       </c>
     </row>
     <row r="32">
@@ -10822,16 +10822,16 @@
         <v>310000</v>
       </c>
       <c r="CC32" t="n">
-        <v>297653.37</v>
+        <v>298699.5377171685</v>
       </c>
       <c r="CD32" t="n">
-        <v>12346.63</v>
+        <v>11300.46228283155</v>
       </c>
       <c r="CE32" t="n">
-        <v>12346.63</v>
+        <v>11300.46228283155</v>
       </c>
       <c r="CF32" t="n">
-        <v>3.982783870967743</v>
+        <v>3.645310413816628</v>
       </c>
     </row>
     <row r="33">
@@ -11150,16 +11150,16 @@
         <v>130000</v>
       </c>
       <c r="CC33" t="n">
-        <v>119782</v>
+        <v>120170.9137647539</v>
       </c>
       <c r="CD33" t="n">
-        <v>10218</v>
+        <v>9829.086235246083</v>
       </c>
       <c r="CE33" t="n">
-        <v>10218</v>
+        <v>9829.086235246083</v>
       </c>
       <c r="CF33" t="n">
-        <v>7.86</v>
+        <v>7.56083556557391</v>
       </c>
     </row>
     <row r="34">
@@ -11474,16 +11474,16 @@
         <v>149900</v>
       </c>
       <c r="CC34" t="n">
-        <v>135072.6</v>
+        <v>134971.9354958758</v>
       </c>
       <c r="CD34" t="n">
-        <v>14827.39999999999</v>
+        <v>14928.0645041242</v>
       </c>
       <c r="CE34" t="n">
-        <v>14827.39999999999</v>
+        <v>14928.0645041242</v>
       </c>
       <c r="CF34" t="n">
-        <v>9.891527685123412</v>
+        <v>9.958682124165573</v>
       </c>
     </row>
     <row r="35">
@@ -11798,16 +11798,16 @@
         <v>140000</v>
       </c>
       <c r="CC35" t="n">
-        <v>156294.52</v>
+        <v>153560.7128091208</v>
       </c>
       <c r="CD35" t="n">
-        <v>-16294.51999999999</v>
+        <v>-13560.71280912077</v>
       </c>
       <c r="CE35" t="n">
-        <v>16294.51999999999</v>
+        <v>13560.71280912077</v>
       </c>
       <c r="CF35" t="n">
-        <v>11.63894285714285</v>
+        <v>9.686223435086266</v>
       </c>
     </row>
     <row r="36">
@@ -12122,16 +12122,16 @@
         <v>174000</v>
       </c>
       <c r="CC36" t="n">
-        <v>178563.06</v>
+        <v>179707.7476568997</v>
       </c>
       <c r="CD36" t="n">
-        <v>-4563.059999999998</v>
+        <v>-5707.747656899737</v>
       </c>
       <c r="CE36" t="n">
-        <v>4563.059999999998</v>
+        <v>5707.747656899737</v>
       </c>
       <c r="CF36" t="n">
-        <v>2.622448275862068</v>
+        <v>3.280314745344676</v>
       </c>
     </row>
     <row r="37">
@@ -12446,16 +12446,16 @@
         <v>374000</v>
       </c>
       <c r="CC37" t="n">
-        <v>349057.86</v>
+        <v>346012.1638769862</v>
       </c>
       <c r="CD37" t="n">
-        <v>24942.14000000001</v>
+        <v>27987.83612301381</v>
       </c>
       <c r="CE37" t="n">
-        <v>24942.14000000001</v>
+        <v>27987.83612301381</v>
       </c>
       <c r="CF37" t="n">
-        <v>6.669021390374335</v>
+        <v>7.483378642517062</v>
       </c>
     </row>
     <row r="38">
@@ -12764,16 +12764,16 @@
         <v>127000</v>
       </c>
       <c r="CC38" t="n">
-        <v>134521</v>
+        <v>132126.658905784</v>
       </c>
       <c r="CD38" t="n">
-        <v>-7521</v>
+        <v>-5126.658905784047</v>
       </c>
       <c r="CE38" t="n">
-        <v>7521</v>
+        <v>5126.658905784047</v>
       </c>
       <c r="CF38" t="n">
-        <v>5.922047244094488</v>
+        <v>4.03673929589295</v>
       </c>
     </row>
     <row r="39">
@@ -13082,16 +13082,16 @@
         <v>177500</v>
       </c>
       <c r="CC39" t="n">
-        <v>169452.32</v>
+        <v>168577.9962567185</v>
       </c>
       <c r="CD39" t="n">
-        <v>8047.679999999993</v>
+        <v>8922.003743281501</v>
       </c>
       <c r="CE39" t="n">
-        <v>8047.679999999993</v>
+        <v>8922.003743281501</v>
       </c>
       <c r="CF39" t="n">
-        <v>4.533904225352109</v>
+        <v>5.026480982130423</v>
       </c>
     </row>
     <row r="40">
@@ -13406,16 +13406,16 @@
         <v>115000</v>
       </c>
       <c r="CC40" t="n">
-        <v>116535.5</v>
+        <v>117995.8704517843</v>
       </c>
       <c r="CD40" t="n">
-        <v>-1535.5</v>
+        <v>-2995.870451784271</v>
       </c>
       <c r="CE40" t="n">
-        <v>1535.5</v>
+        <v>2995.870451784271</v>
       </c>
       <c r="CF40" t="n">
-        <v>1.335217391304348</v>
+        <v>2.605104740681975</v>
       </c>
     </row>
     <row r="41">
@@ -13734,16 +13734,16 @@
         <v>127000</v>
       </c>
       <c r="CC41" t="n">
-        <v>141209.04</v>
+        <v>136968.5450698915</v>
       </c>
       <c r="CD41" t="n">
-        <v>-14209.04000000001</v>
+        <v>-9968.545069891523</v>
       </c>
       <c r="CE41" t="n">
-        <v>14209.04000000001</v>
+        <v>9968.545069891523</v>
       </c>
       <c r="CF41" t="n">
-        <v>11.18822047244095</v>
+        <v>7.849248086528758</v>
       </c>
     </row>
     <row r="42">
@@ -14058,16 +14058,16 @@
         <v>89471</v>
       </c>
       <c r="CC42" t="n">
-        <v>118055.02</v>
+        <v>116355.0536847521</v>
       </c>
       <c r="CD42" t="n">
-        <v>-28584.02</v>
+        <v>-26884.05368475206</v>
       </c>
       <c r="CE42" t="n">
-        <v>28584.02</v>
+        <v>26884.05368475206</v>
       </c>
       <c r="CF42" t="n">
-        <v>31.94780431648244</v>
+        <v>30.04778496356591</v>
       </c>
     </row>
     <row r="43">
@@ -14382,16 +14382,16 @@
         <v>270000</v>
       </c>
       <c r="CC43" t="n">
-        <v>246519.4</v>
+        <v>251531.3426213611</v>
       </c>
       <c r="CD43" t="n">
-        <v>23480.60000000001</v>
+        <v>18468.65737863895</v>
       </c>
       <c r="CE43" t="n">
-        <v>23480.60000000001</v>
+        <v>18468.65737863895</v>
       </c>
       <c r="CF43" t="n">
-        <v>8.69651851851852</v>
+        <v>6.840243473569981</v>
       </c>
     </row>
     <row r="44">
@@ -14706,16 +14706,16 @@
         <v>152000</v>
       </c>
       <c r="CC44" t="n">
-        <v>145126.78</v>
+        <v>147517.1730236814</v>
       </c>
       <c r="CD44" t="n">
-        <v>6873.220000000001</v>
+        <v>4482.826976318553</v>
       </c>
       <c r="CE44" t="n">
-        <v>6873.220000000001</v>
+        <v>4482.826976318553</v>
       </c>
       <c r="CF44" t="n">
-        <v>4.521855263157896</v>
+        <v>2.949228273893785</v>
       </c>
     </row>
     <row r="45">
@@ -15024,16 +15024,16 @@
         <v>135000</v>
       </c>
       <c r="CC45" t="n">
-        <v>137721.5</v>
+        <v>136662.1930184665</v>
       </c>
       <c r="CD45" t="n">
-        <v>-2721.5</v>
+        <v>-1662.193018466525</v>
       </c>
       <c r="CE45" t="n">
-        <v>2721.5</v>
+        <v>1662.193018466525</v>
       </c>
       <c r="CF45" t="n">
-        <v>2.015925925925926</v>
+        <v>1.231254087752982</v>
       </c>
     </row>
     <row r="46">
@@ -15348,16 +15348,16 @@
         <v>180000</v>
       </c>
       <c r="CC46" t="n">
-        <v>209327.86</v>
+        <v>211350.5930837096</v>
       </c>
       <c r="CD46" t="n">
-        <v>-29327.85999999999</v>
+        <v>-31350.59308370957</v>
       </c>
       <c r="CE46" t="n">
-        <v>29327.85999999999</v>
+        <v>31350.59308370957</v>
       </c>
       <c r="CF46" t="n">
-        <v>16.29325555555555</v>
+        <v>17.41699615761643</v>
       </c>
     </row>
     <row r="47">
@@ -15668,16 +15668,16 @@
         <v>118500</v>
       </c>
       <c r="CC47" t="n">
-        <v>118631</v>
+        <v>118401.0244112704</v>
       </c>
       <c r="CD47" t="n">
-        <v>-131</v>
+        <v>98.97558872964873</v>
       </c>
       <c r="CE47" t="n">
-        <v>131</v>
+        <v>98.97558872964873</v>
       </c>
       <c r="CF47" t="n">
-        <v>0.1105485232067511</v>
+        <v>0.08352370356932383</v>
       </c>
     </row>
     <row r="48">
@@ -15992,16 +15992,16 @@
         <v>367294</v>
       </c>
       <c r="CC48" t="n">
-        <v>411164.66</v>
+        <v>399569.2051525337</v>
       </c>
       <c r="CD48" t="n">
-        <v>-43870.65999999997</v>
+        <v>-32275.20515253372</v>
       </c>
       <c r="CE48" t="n">
-        <v>43870.65999999997</v>
+        <v>32275.20515253372</v>
       </c>
       <c r="CF48" t="n">
-        <v>11.94428986043877</v>
+        <v>8.787294416062805</v>
       </c>
     </row>
     <row r="49">
@@ -16320,16 +16320,16 @@
         <v>40000</v>
       </c>
       <c r="CC49" t="n">
-        <v>96538.5</v>
+        <v>96367.55779157029</v>
       </c>
       <c r="CD49" t="n">
-        <v>-56538.5</v>
+        <v>-56367.55779157029</v>
       </c>
       <c r="CE49" t="n">
-        <v>56538.5</v>
+        <v>56367.55779157029</v>
       </c>
       <c r="CF49" t="n">
-        <v>141.34625</v>
+        <v>140.9188944789257</v>
       </c>
     </row>
     <row r="50">
@@ -16640,16 +16640,16 @@
         <v>175900</v>
       </c>
       <c r="CC50" t="n">
-        <v>173277.85</v>
+        <v>173778.0218364276</v>
       </c>
       <c r="CD50" t="n">
-        <v>2622.149999999994</v>
+        <v>2121.978163572407</v>
       </c>
       <c r="CE50" t="n">
-        <v>2622.149999999994</v>
+        <v>2121.978163572407</v>
       </c>
       <c r="CF50" t="n">
-        <v>1.490704945992038</v>
+        <v>1.206354840007053</v>
       </c>
     </row>
     <row r="51">
@@ -16960,16 +16960,16 @@
         <v>120000</v>
       </c>
       <c r="CC51" t="n">
-        <v>122783.5</v>
+        <v>120742.8710193811</v>
       </c>
       <c r="CD51" t="n">
-        <v>-2783.5</v>
+        <v>-742.871019381113</v>
       </c>
       <c r="CE51" t="n">
-        <v>2783.5</v>
+        <v>742.871019381113</v>
       </c>
       <c r="CF51" t="n">
-        <v>2.319583333333333</v>
+        <v>0.6190591828175942</v>
       </c>
     </row>
     <row r="52">
@@ -17288,16 +17288,16 @@
         <v>119000</v>
       </c>
       <c r="CC52" t="n">
-        <v>111153.5</v>
+        <v>113265.8307050216</v>
       </c>
       <c r="CD52" t="n">
-        <v>7846.5</v>
+        <v>5734.169294978405</v>
       </c>
       <c r="CE52" t="n">
-        <v>7846.5</v>
+        <v>5734.169294978405</v>
       </c>
       <c r="CF52" t="n">
-        <v>6.593697478991596</v>
+        <v>4.818629659645718</v>
       </c>
     </row>
     <row r="53">
@@ -17608,16 +17608,16 @@
         <v>133000</v>
       </c>
       <c r="CC53" t="n">
-        <v>153996.6</v>
+        <v>151850.4193045299</v>
       </c>
       <c r="CD53" t="n">
-        <v>-20996.60000000001</v>
+        <v>-18850.4193045299</v>
       </c>
       <c r="CE53" t="n">
-        <v>20996.60000000001</v>
+        <v>18850.4193045299</v>
       </c>
       <c r="CF53" t="n">
-        <v>15.78691729323309</v>
+        <v>14.17324759739091</v>
       </c>
     </row>
     <row r="54">
@@ -17928,16 +17928,16 @@
         <v>201000</v>
       </c>
       <c r="CC54" t="n">
-        <v>233237.97</v>
+        <v>234942.388527533</v>
       </c>
       <c r="CD54" t="n">
-        <v>-32237.97</v>
+        <v>-33942.38852753295</v>
       </c>
       <c r="CE54" t="n">
-        <v>32237.97</v>
+        <v>33942.38852753295</v>
       </c>
       <c r="CF54" t="n">
-        <v>16.03879104477612</v>
+        <v>16.88676046145918</v>
       </c>
     </row>
     <row r="55">
@@ -18250,16 +18250,16 @@
         <v>180000</v>
       </c>
       <c r="CC55" t="n">
-        <v>173454.19</v>
+        <v>169523.5022503228</v>
       </c>
       <c r="CD55" t="n">
-        <v>6545.809999999998</v>
+        <v>10476.49774967716</v>
       </c>
       <c r="CE55" t="n">
-        <v>6545.809999999998</v>
+        <v>10476.49774967716</v>
       </c>
       <c r="CF55" t="n">
-        <v>3.63656111111111</v>
+        <v>5.820276527598423</v>
       </c>
     </row>
     <row r="56">
@@ -18556,16 +18556,16 @@
         <v>85000</v>
       </c>
       <c r="CC56" t="n">
-        <v>106865.25</v>
+        <v>106567.0411045947</v>
       </c>
       <c r="CD56" t="n">
-        <v>-21865.25</v>
+        <v>-21567.04110459465</v>
       </c>
       <c r="CE56" t="n">
-        <v>21865.25</v>
+        <v>21567.04110459465</v>
       </c>
       <c r="CF56" t="n">
-        <v>25.72382352941177</v>
+        <v>25.37298953481724</v>
       </c>
     </row>
     <row r="57">
@@ -18880,16 +18880,16 @@
         <v>79500</v>
       </c>
       <c r="CC57" t="n">
-        <v>114214.5</v>
+        <v>114488.4965229463</v>
       </c>
       <c r="CD57" t="n">
-        <v>-34714.5</v>
+        <v>-34988.49652294628</v>
       </c>
       <c r="CE57" t="n">
-        <v>34714.5</v>
+        <v>34988.49652294628</v>
       </c>
       <c r="CF57" t="n">
-        <v>43.66603773584906</v>
+        <v>44.0106874502469</v>
       </c>
     </row>
     <row r="58">
@@ -19202,16 +19202,16 @@
         <v>228500</v>
       </c>
       <c r="CC58" t="n">
-        <v>267872.86</v>
+        <v>267488.1953825968</v>
       </c>
       <c r="CD58" t="n">
-        <v>-39372.85999999999</v>
+        <v>-38988.19538259681</v>
       </c>
       <c r="CE58" t="n">
-        <v>39372.85999999999</v>
+        <v>38988.19538259681</v>
       </c>
       <c r="CF58" t="n">
-        <v>17.23101094091903</v>
+        <v>17.0626675634997</v>
       </c>
     </row>
     <row r="59">
@@ -19524,16 +19524,16 @@
         <v>275000</v>
       </c>
       <c r="CC59" t="n">
-        <v>278939.59</v>
+        <v>277469.4069897784</v>
       </c>
       <c r="CD59" t="n">
-        <v>-3939.590000000026</v>
+        <v>-2469.406989778392</v>
       </c>
       <c r="CE59" t="n">
-        <v>3939.590000000026</v>
+        <v>2469.406989778392</v>
       </c>
       <c r="CF59" t="n">
-        <v>1.432578181818191</v>
+        <v>0.8979661781012335</v>
       </c>
     </row>
     <row r="60">
@@ -19850,16 +19850,16 @@
         <v>150000</v>
       </c>
       <c r="CC60" t="n">
-        <v>166334.5</v>
+        <v>166948.6832349962</v>
       </c>
       <c r="CD60" t="n">
-        <v>-16334.5</v>
+        <v>-16948.68323499619</v>
       </c>
       <c r="CE60" t="n">
-        <v>16334.5</v>
+        <v>16948.68323499619</v>
       </c>
       <c r="CF60" t="n">
-        <v>10.88966666666667</v>
+        <v>11.29912215666413</v>
       </c>
     </row>
     <row r="61">
@@ -20156,16 +20156,16 @@
         <v>104000</v>
       </c>
       <c r="CC61" t="n">
-        <v>135447.73</v>
+        <v>138359.4201072456</v>
       </c>
       <c r="CD61" t="n">
-        <v>-31447.73000000001</v>
+        <v>-34359.42010724562</v>
       </c>
       <c r="CE61" t="n">
-        <v>31447.73000000001</v>
+        <v>34359.42010724562</v>
       </c>
       <c r="CF61" t="n">
-        <v>30.23820192307694</v>
+        <v>33.03790394927464</v>
       </c>
     </row>
     <row r="62">
@@ -20480,16 +20480,16 @@
         <v>314813</v>
       </c>
       <c r="CC62" t="n">
-        <v>348261.24</v>
+        <v>341770.6920569616</v>
       </c>
       <c r="CD62" t="n">
-        <v>-33448.23999999999</v>
+        <v>-26957.69205696165</v>
       </c>
       <c r="CE62" t="n">
-        <v>33448.23999999999</v>
+        <v>26957.69205696165</v>
       </c>
       <c r="CF62" t="n">
-        <v>10.6247963076493</v>
+        <v>8.563080958207459</v>
       </c>
     </row>
     <row r="63">
@@ -20798,16 +20798,16 @@
         <v>128500</v>
       </c>
       <c r="CC63" t="n">
-        <v>137419.6</v>
+        <v>136708.3387026908</v>
       </c>
       <c r="CD63" t="n">
-        <v>-8919.600000000006</v>
+        <v>-8208.338702690759</v>
       </c>
       <c r="CE63" t="n">
-        <v>8919.600000000006</v>
+        <v>8208.338702690759</v>
       </c>
       <c r="CF63" t="n">
-        <v>6.941322957198448</v>
+        <v>6.387812219992808</v>
       </c>
     </row>
     <row r="64">
@@ -21100,16 +21100,16 @@
         <v>130000</v>
       </c>
       <c r="CC64" t="n">
-        <v>133249.22</v>
+        <v>131318.799829167</v>
       </c>
       <c r="CD64" t="n">
-        <v>-3249.220000000001</v>
+        <v>-1318.799829167023</v>
       </c>
       <c r="CE64" t="n">
-        <v>3249.220000000001</v>
+        <v>1318.799829167023</v>
       </c>
       <c r="CF64" t="n">
-        <v>2.499400000000001</v>
+        <v>1.014461407051556</v>
       </c>
     </row>
     <row r="65">
@@ -21428,16 +21428,16 @@
         <v>243000</v>
       </c>
       <c r="CC65" t="n">
-        <v>199101.41</v>
+        <v>205925.5547237801</v>
       </c>
       <c r="CD65" t="n">
-        <v>43898.59</v>
+        <v>37074.44527621992</v>
       </c>
       <c r="CE65" t="n">
-        <v>43898.59</v>
+        <v>37074.44527621992</v>
       </c>
       <c r="CF65" t="n">
-        <v>18.0652633744856</v>
+        <v>15.25697336469955</v>
       </c>
     </row>
     <row r="66">
@@ -21748,16 +21748,16 @@
         <v>109500</v>
       </c>
       <c r="CC66" t="n">
-        <v>114417.25</v>
+        <v>114477.8793710881</v>
       </c>
       <c r="CD66" t="n">
-        <v>-4917.25</v>
+        <v>-4977.879371088115</v>
       </c>
       <c r="CE66" t="n">
-        <v>4917.25</v>
+        <v>4977.879371088115</v>
       </c>
       <c r="CF66" t="n">
-        <v>4.490639269406393</v>
+        <v>4.546008558071338</v>
       </c>
     </row>
     <row r="67">
@@ -22068,16 +22068,16 @@
         <v>133000</v>
       </c>
       <c r="CC67" t="n">
-        <v>132093.35</v>
+        <v>131559.3348651607</v>
       </c>
       <c r="CD67" t="n">
-        <v>906.6499999999942</v>
+        <v>1440.665134839335</v>
       </c>
       <c r="CE67" t="n">
-        <v>906.6499999999942</v>
+        <v>1440.665134839335</v>
       </c>
       <c r="CF67" t="n">
-        <v>0.6816917293233039</v>
+        <v>1.083206868300252</v>
       </c>
     </row>
     <row r="68">
@@ -22386,16 +22386,16 @@
         <v>194500</v>
       </c>
       <c r="CC68" t="n">
-        <v>213074.63</v>
+        <v>207991.0766976178</v>
       </c>
       <c r="CD68" t="n">
-        <v>-18574.63</v>
+        <v>-13491.0766976178</v>
       </c>
       <c r="CE68" t="n">
-        <v>18574.63</v>
+        <v>13491.0766976178</v>
       </c>
       <c r="CF68" t="n">
-        <v>9.549938303341905</v>
+        <v>6.936286219854909</v>
       </c>
     </row>
     <row r="69">
@@ -22708,16 +22708,16 @@
         <v>271000</v>
       </c>
       <c r="CC69" t="n">
-        <v>286662.45</v>
+        <v>285852.5916046458</v>
       </c>
       <c r="CD69" t="n">
-        <v>-15662.45000000001</v>
+        <v>-14852.59160464577</v>
       </c>
       <c r="CE69" t="n">
-        <v>15662.45000000001</v>
+        <v>14852.59160464577</v>
       </c>
       <c r="CF69" t="n">
-        <v>5.779501845018455</v>
+        <v>5.480661108725378</v>
       </c>
     </row>
     <row r="70">
@@ -23040,16 +23040,16 @@
         <v>131400</v>
       </c>
       <c r="CC70" t="n">
-        <v>131029.25</v>
+        <v>131791.6757411357</v>
       </c>
       <c r="CD70" t="n">
-        <v>370.75</v>
+        <v>-391.6757411356957</v>
       </c>
       <c r="CE70" t="n">
-        <v>370.75</v>
+        <v>391.6757411356957</v>
       </c>
       <c r="CF70" t="n">
-        <v>0.2821537290715373</v>
+        <v>0.2980789506359937</v>
       </c>
     </row>
     <row r="71">
@@ -23364,16 +23364,16 @@
         <v>81000</v>
       </c>
       <c r="CC71" t="n">
-        <v>110225.5</v>
+        <v>109589.2960743296</v>
       </c>
       <c r="CD71" t="n">
-        <v>-29225.5</v>
+        <v>-28589.29607432961</v>
       </c>
       <c r="CE71" t="n">
-        <v>29225.5</v>
+        <v>28589.29607432961</v>
       </c>
       <c r="CF71" t="n">
-        <v>36.08086419753086</v>
+        <v>35.29542725225878</v>
       </c>
     </row>
     <row r="72">
@@ -23688,16 +23688,16 @@
         <v>140000</v>
       </c>
       <c r="CC72" t="n">
-        <v>148322.75</v>
+        <v>148982.2830318806</v>
       </c>
       <c r="CD72" t="n">
-        <v>-8322.75</v>
+        <v>-8982.283031880623</v>
       </c>
       <c r="CE72" t="n">
-        <v>8322.75</v>
+        <v>8982.283031880623</v>
       </c>
       <c r="CF72" t="n">
-        <v>5.944821428571428</v>
+        <v>6.415916451343302</v>
       </c>
     </row>
     <row r="73">
@@ -24012,16 +24012,16 @@
         <v>181000</v>
       </c>
       <c r="CC73" t="n">
-        <v>179231.77</v>
+        <v>179467.5243709022</v>
       </c>
       <c r="CD73" t="n">
-        <v>1768.23000000001</v>
+        <v>1532.475629097782</v>
       </c>
       <c r="CE73" t="n">
-        <v>1768.23000000001</v>
+        <v>1532.475629097782</v>
       </c>
       <c r="CF73" t="n">
-        <v>0.9769226519337074</v>
+        <v>0.8466716182860674</v>
       </c>
     </row>
     <row r="74">
@@ -24336,16 +24336,16 @@
         <v>360000</v>
       </c>
       <c r="CC74" t="n">
-        <v>344365.2</v>
+        <v>352864.2547476437</v>
       </c>
       <c r="CD74" t="n">
-        <v>15634.79999999999</v>
+        <v>7135.745252356282</v>
       </c>
       <c r="CE74" t="n">
-        <v>15634.79999999999</v>
+        <v>7135.745252356282</v>
       </c>
       <c r="CF74" t="n">
-        <v>4.342999999999996</v>
+        <v>1.982151458987856</v>
       </c>
     </row>
     <row r="75">
@@ -24660,16 +24660,16 @@
         <v>178000</v>
       </c>
       <c r="CC75" t="n">
-        <v>179181.75</v>
+        <v>179096.4384360313</v>
       </c>
       <c r="CD75" t="n">
-        <v>-1181.75</v>
+        <v>-1096.438436031312</v>
       </c>
       <c r="CE75" t="n">
-        <v>1181.75</v>
+        <v>1096.438436031312</v>
       </c>
       <c r="CF75" t="n">
-        <v>0.6639044943820225</v>
+        <v>0.6159766494557936</v>
       </c>
     </row>
     <row r="76">
@@ -24978,16 +24978,16 @@
         <v>145000</v>
       </c>
       <c r="CC76" t="n">
-        <v>120720</v>
+        <v>119583.7706615444</v>
       </c>
       <c r="CD76" t="n">
-        <v>24280</v>
+        <v>25416.22933845555</v>
       </c>
       <c r="CE76" t="n">
-        <v>24280</v>
+        <v>25416.22933845555</v>
       </c>
       <c r="CF76" t="n">
-        <v>16.7448275862069</v>
+        <v>17.52843402652107</v>
       </c>
     </row>
     <row r="77">
@@ -25302,16 +25302,16 @@
         <v>125500</v>
       </c>
       <c r="CC77" t="n">
-        <v>110118</v>
+        <v>108006.413276085</v>
       </c>
       <c r="CD77" t="n">
-        <v>15382</v>
+        <v>17493.58672391497</v>
       </c>
       <c r="CE77" t="n">
-        <v>15382</v>
+        <v>17493.58672391497</v>
       </c>
       <c r="CF77" t="n">
-        <v>12.25657370517928</v>
+        <v>13.93911292742228</v>
       </c>
     </row>
     <row r="78">
@@ -25626,16 +25626,16 @@
         <v>254000</v>
       </c>
       <c r="CC78" t="n">
-        <v>236059.31</v>
+        <v>238630.3854592624</v>
       </c>
       <c r="CD78" t="n">
-        <v>17940.69</v>
+        <v>15369.61454073765</v>
       </c>
       <c r="CE78" t="n">
-        <v>17940.69</v>
+        <v>15369.61454073765</v>
       </c>
       <c r="CF78" t="n">
-        <v>7.063263779527559</v>
+        <v>6.051029346747105</v>
       </c>
     </row>
     <row r="79">
@@ -25950,16 +25950,16 @@
         <v>169990</v>
       </c>
       <c r="CC79" t="n">
-        <v>178276.25</v>
+        <v>176804.8735377844</v>
       </c>
       <c r="CD79" t="n">
-        <v>-8286.25</v>
+        <v>-6814.873537784355</v>
       </c>
       <c r="CE79" t="n">
-        <v>8286.25</v>
+        <v>6814.873537784355</v>
       </c>
       <c r="CF79" t="n">
-        <v>4.8745514442026</v>
+        <v>4.008984962518004</v>
       </c>
     </row>
     <row r="80">
@@ -26272,16 +26272,16 @@
         <v>196000</v>
       </c>
       <c r="CC80" t="n">
-        <v>189933.78</v>
+        <v>192003.0594878126</v>
       </c>
       <c r="CD80" t="n">
-        <v>6066.220000000001</v>
+        <v>3996.940512187401</v>
       </c>
       <c r="CE80" t="n">
-        <v>6066.220000000001</v>
+        <v>3996.940512187401</v>
       </c>
       <c r="CF80" t="n">
-        <v>3.095010204081633</v>
+        <v>2.039255363360919</v>
       </c>
     </row>
     <row r="81">
@@ -26592,16 +26592,16 @@
         <v>105900</v>
       </c>
       <c r="CC81" t="n">
-        <v>119969</v>
+        <v>120721.3560433388</v>
       </c>
       <c r="CD81" t="n">
-        <v>-14069</v>
+        <v>-14821.35604333885</v>
       </c>
       <c r="CE81" t="n">
-        <v>14069</v>
+        <v>14821.35604333885</v>
       </c>
       <c r="CF81" t="n">
-        <v>13.2851746931067</v>
+        <v>13.9956147718025</v>
       </c>
     </row>
     <row r="82">
@@ -26920,16 +26920,16 @@
         <v>187750</v>
       </c>
       <c r="CC82" t="n">
-        <v>190208.34</v>
+        <v>190997.8177345879</v>
       </c>
       <c r="CD82" t="n">
-        <v>-2458.339999999997</v>
+        <v>-3247.817734587908</v>
       </c>
       <c r="CE82" t="n">
-        <v>2458.339999999997</v>
+        <v>3247.817734587908</v>
       </c>
       <c r="CF82" t="n">
-        <v>1.309368841544605</v>
+        <v>1.72986297448091</v>
       </c>
     </row>
     <row r="83">
@@ -27240,16 +27240,16 @@
         <v>206300</v>
       </c>
       <c r="CC83" t="n">
-        <v>188663.9</v>
+        <v>189882.0253191712</v>
       </c>
       <c r="CD83" t="n">
-        <v>17636.10000000001</v>
+        <v>16417.97468082877</v>
       </c>
       <c r="CE83" t="n">
-        <v>17636.10000000001</v>
+        <v>16417.97468082877</v>
       </c>
       <c r="CF83" t="n">
-        <v>8.548763936015515</v>
+        <v>7.958300863222867</v>
       </c>
     </row>
     <row r="84">
@@ -27564,16 +27564,16 @@
         <v>125500</v>
       </c>
       <c r="CC84" t="n">
-        <v>116767</v>
+        <v>117220.4718094218</v>
       </c>
       <c r="CD84" t="n">
-        <v>8733</v>
+        <v>8279.528190578218</v>
       </c>
       <c r="CE84" t="n">
-        <v>8733</v>
+        <v>8279.528190578218</v>
       </c>
       <c r="CF84" t="n">
-        <v>6.958565737051793</v>
+        <v>6.597233617990611</v>
       </c>
     </row>
     <row r="85">
@@ -27886,16 +27886,16 @@
         <v>205000</v>
       </c>
       <c r="CC85" t="n">
-        <v>234366.79</v>
+        <v>233215.6099156755</v>
       </c>
       <c r="CD85" t="n">
-        <v>-29366.79000000001</v>
+        <v>-28215.60991567551</v>
       </c>
       <c r="CE85" t="n">
-        <v>29366.79000000001</v>
+        <v>28215.60991567551</v>
       </c>
       <c r="CF85" t="n">
-        <v>14.32526341463415</v>
+        <v>13.76371215398805</v>
       </c>
     </row>
     <row r="86">
@@ -28208,16 +28208,16 @@
         <v>188000</v>
       </c>
       <c r="CC86" t="n">
-        <v>184044.01</v>
+        <v>184029.828165676</v>
       </c>
       <c r="CD86" t="n">
-        <v>3955.989999999991</v>
+        <v>3970.171834323963</v>
       </c>
       <c r="CE86" t="n">
-        <v>3955.989999999991</v>
+        <v>3970.171834323963</v>
       </c>
       <c r="CF86" t="n">
-        <v>2.104249999999995</v>
+        <v>2.111793528895725</v>
       </c>
     </row>
     <row r="87">
@@ -28532,16 +28532,16 @@
         <v>239500</v>
       </c>
       <c r="CC87" t="n">
-        <v>236764.95</v>
+        <v>236934.4945876746</v>
       </c>
       <c r="CD87" t="n">
-        <v>2735.049999999988</v>
+        <v>2565.505412325409</v>
       </c>
       <c r="CE87" t="n">
-        <v>2735.049999999988</v>
+        <v>2565.505412325409</v>
       </c>
       <c r="CF87" t="n">
-        <v>1.141983298538617</v>
+        <v>1.071192238966768</v>
       </c>
     </row>
     <row r="88">
@@ -28852,16 +28852,16 @@
         <v>197000</v>
       </c>
       <c r="CC88" t="n">
-        <v>188025.53</v>
+        <v>190867.6605439152</v>
       </c>
       <c r="CD88" t="n">
-        <v>8974.470000000001</v>
+        <v>6132.339456084825</v>
       </c>
       <c r="CE88" t="n">
-        <v>8974.470000000001</v>
+        <v>6132.339456084825</v>
       </c>
       <c r="CF88" t="n">
-        <v>4.555568527918783</v>
+        <v>3.112862668063363</v>
       </c>
     </row>
     <row r="89">
@@ -29174,16 +29174,16 @@
         <v>158000</v>
       </c>
       <c r="CC89" t="n">
-        <v>145762</v>
+        <v>146657.21590008</v>
       </c>
       <c r="CD89" t="n">
-        <v>12238</v>
+        <v>11342.78409992001</v>
       </c>
       <c r="CE89" t="n">
-        <v>12238</v>
+        <v>11342.78409992001</v>
       </c>
       <c r="CF89" t="n">
-        <v>7.745569620253165</v>
+        <v>7.178977278430388</v>
       </c>
     </row>
     <row r="90">
@@ -29498,16 +29498,16 @@
         <v>127500</v>
       </c>
       <c r="CC90" t="n">
-        <v>121890.04</v>
+        <v>122834.677684746</v>
       </c>
       <c r="CD90" t="n">
-        <v>5609.960000000006</v>
+        <v>4665.322315254045</v>
       </c>
       <c r="CE90" t="n">
-        <v>5609.960000000006</v>
+        <v>4665.322315254045</v>
       </c>
       <c r="CF90" t="n">
-        <v>4.399968627450986</v>
+        <v>3.659076325689447</v>
       </c>
     </row>
     <row r="91">
@@ -29822,16 +29822,16 @@
         <v>315500</v>
       </c>
       <c r="CC91" t="n">
-        <v>317682.95</v>
+        <v>319843.151996045</v>
       </c>
       <c r="CD91" t="n">
-        <v>-2182.950000000012</v>
+        <v>-4343.151996045024</v>
       </c>
       <c r="CE91" t="n">
-        <v>2182.950000000012</v>
+        <v>4343.151996045024</v>
       </c>
       <c r="CF91" t="n">
-        <v>0.691901743264663</v>
+        <v>1.376593342645016</v>
       </c>
     </row>
     <row r="92">
@@ -30144,16 +30144,16 @@
         <v>115000</v>
       </c>
       <c r="CC92" t="n">
-        <v>115299.62</v>
+        <v>114271.6554553393</v>
       </c>
       <c r="CD92" t="n">
-        <v>-299.6199999999953</v>
+        <v>728.3445446607075</v>
       </c>
       <c r="CE92" t="n">
-        <v>299.6199999999953</v>
+        <v>728.3445446607075</v>
       </c>
       <c r="CF92" t="n">
-        <v>0.2605391304347786</v>
+        <v>0.6333430823136587</v>
       </c>
     </row>
     <row r="93">
@@ -30466,16 +30466,16 @@
         <v>128000</v>
       </c>
       <c r="CC93" t="n">
-        <v>140765.32</v>
+        <v>140894.2389745397</v>
       </c>
       <c r="CD93" t="n">
-        <v>-12765.32000000001</v>
+        <v>-12894.23897453971</v>
       </c>
       <c r="CE93" t="n">
-        <v>12765.32000000001</v>
+        <v>12894.23897453971</v>
       </c>
       <c r="CF93" t="n">
-        <v>9.972906250000005</v>
+        <v>10.07362419885915</v>
       </c>
     </row>
     <row r="94">
@@ -30788,16 +30788,16 @@
         <v>163500</v>
       </c>
       <c r="CC94" t="n">
-        <v>179390</v>
+        <v>178770.6799370018</v>
       </c>
       <c r="CD94" t="n">
-        <v>-15890</v>
+        <v>-15270.67993700175</v>
       </c>
       <c r="CE94" t="n">
-        <v>15890</v>
+        <v>15270.67993700175</v>
       </c>
       <c r="CF94" t="n">
-        <v>9.718654434250764</v>
+        <v>9.33986540489404</v>
       </c>
     </row>
     <row r="95">
@@ -31108,16 +31108,16 @@
         <v>68400</v>
       </c>
       <c r="CC95" t="n">
-        <v>108815.5</v>
+        <v>108032.7799065057</v>
       </c>
       <c r="CD95" t="n">
-        <v>-40415.5</v>
+        <v>-39632.77990650573</v>
       </c>
       <c r="CE95" t="n">
-        <v>40415.5</v>
+        <v>39632.77990650573</v>
       </c>
       <c r="CF95" t="n">
-        <v>59.08698830409357</v>
+        <v>57.94266068202592</v>
       </c>
     </row>
     <row r="96">
@@ -31430,16 +31430,16 @@
         <v>161500</v>
       </c>
       <c r="CC96" t="n">
-        <v>157884.82</v>
+        <v>159040.7903266423</v>
       </c>
       <c r="CD96" t="n">
-        <v>3615.179999999993</v>
+        <v>2459.209673357662</v>
       </c>
       <c r="CE96" t="n">
-        <v>3615.179999999993</v>
+        <v>2459.209673357662</v>
       </c>
       <c r="CF96" t="n">
-        <v>2.238501547987612</v>
+        <v>1.522730447899481</v>
       </c>
     </row>
     <row r="97">
@@ -31754,16 +31754,16 @@
         <v>172500</v>
       </c>
       <c r="CC97" t="n">
-        <v>162096.83</v>
+        <v>162864.234880564</v>
       </c>
       <c r="CD97" t="n">
-        <v>10403.17000000001</v>
+        <v>9635.765119435993</v>
       </c>
       <c r="CE97" t="n">
-        <v>10403.17000000001</v>
+        <v>9635.765119435993</v>
       </c>
       <c r="CF97" t="n">
-        <v>6.030823188405805</v>
+        <v>5.585950793875938</v>
       </c>
     </row>
     <row r="98">
@@ -32060,16 +32060,16 @@
         <v>103200</v>
       </c>
       <c r="CC98" t="n">
-        <v>95564.5</v>
+        <v>97648.11714648447</v>
       </c>
       <c r="CD98" t="n">
-        <v>7635.5</v>
+        <v>5551.882853515533</v>
       </c>
       <c r="CE98" t="n">
-        <v>7635.5</v>
+        <v>5551.882853515533</v>
       </c>
       <c r="CF98" t="n">
-        <v>7.398740310077518</v>
+        <v>5.379731447204975</v>
       </c>
     </row>
     <row r="99">
@@ -32380,16 +32380,16 @@
         <v>204900</v>
       </c>
       <c r="CC99" t="n">
-        <v>220298.7</v>
+        <v>219693.7396842899</v>
       </c>
       <c r="CD99" t="n">
-        <v>-15398.70000000001</v>
+        <v>-14793.7396842899</v>
       </c>
       <c r="CE99" t="n">
-        <v>15398.70000000001</v>
+        <v>14793.7396842899</v>
       </c>
       <c r="CF99" t="n">
-        <v>7.515226939970724</v>
+        <v>7.219980324202002</v>
       </c>
     </row>
     <row r="100">
@@ -32700,16 +32700,16 @@
         <v>145000</v>
       </c>
       <c r="CC100" t="n">
-        <v>144046.5</v>
+        <v>144879.3559928754</v>
       </c>
       <c r="CD100" t="n">
-        <v>953.5</v>
+        <v>120.644007124647</v>
       </c>
       <c r="CE100" t="n">
-        <v>953.5</v>
+        <v>120.644007124647</v>
       </c>
       <c r="CF100" t="n">
-        <v>0.6575862068965518</v>
+        <v>0.08320276353423933</v>
       </c>
     </row>
     <row r="101">
@@ -33020,16 +33020,16 @@
         <v>262500</v>
       </c>
       <c r="CC101" t="n">
-        <v>266906.36</v>
+        <v>268270.4060429557</v>
       </c>
       <c r="CD101" t="n">
-        <v>-4406.359999999986</v>
+        <v>-5770.406042955699</v>
       </c>
       <c r="CE101" t="n">
-        <v>4406.359999999986</v>
+        <v>5770.406042955699</v>
       </c>
       <c r="CF101" t="n">
-        <v>1.678613333333328</v>
+        <v>2.198249921125981</v>
       </c>
     </row>
     <row r="102">
@@ -33344,16 +33344,16 @@
         <v>154000</v>
       </c>
       <c r="CC102" t="n">
-        <v>146608.07</v>
+        <v>148947.272191377</v>
       </c>
       <c r="CD102" t="n">
-        <v>7391.929999999993</v>
+        <v>5052.727808622993</v>
       </c>
       <c r="CE102" t="n">
-        <v>7391.929999999993</v>
+        <v>5052.727808622993</v>
       </c>
       <c r="CF102" t="n">
-        <v>4.799954545454541</v>
+        <v>3.280992083521424</v>
       </c>
     </row>
     <row r="103">
@@ -33668,16 +33668,16 @@
         <v>127000</v>
       </c>
       <c r="CC103" t="n">
-        <v>125959.5</v>
+        <v>126217.3439937832</v>
       </c>
       <c r="CD103" t="n">
-        <v>1040.5</v>
+        <v>782.6560062167846</v>
       </c>
       <c r="CE103" t="n">
-        <v>1040.5</v>
+        <v>782.6560062167846</v>
       </c>
       <c r="CF103" t="n">
-        <v>0.8192913385826771</v>
+        <v>0.6162645718242399</v>
       </c>
     </row>
     <row r="104">
@@ -33978,16 +33978,16 @@
         <v>200500</v>
       </c>
       <c r="CC104" t="n">
-        <v>171808.42</v>
+        <v>177080.3116858793</v>
       </c>
       <c r="CD104" t="n">
-        <v>28691.57999999999</v>
+        <v>23419.68831412069</v>
       </c>
       <c r="CE104" t="n">
-        <v>28691.57999999999</v>
+        <v>23419.68831412069</v>
       </c>
       <c r="CF104" t="n">
-        <v>14.31001496259351</v>
+        <v>11.68064255068364</v>
       </c>
     </row>
     <row r="105">
@@ -34296,16 +34296,16 @@
         <v>144000</v>
       </c>
       <c r="CC105" t="n">
-        <v>140219.9</v>
+        <v>140210.7755084976</v>
       </c>
       <c r="CD105" t="n">
-        <v>3780.100000000006</v>
+        <v>3789.22449150242</v>
       </c>
       <c r="CE105" t="n">
-        <v>3780.100000000006</v>
+        <v>3789.22449150242</v>
       </c>
       <c r="CF105" t="n">
-        <v>2.625069444444449</v>
+        <v>2.631405896876681</v>
       </c>
     </row>
     <row r="106">
@@ -34620,16 +34620,16 @@
         <v>280000</v>
       </c>
       <c r="CC106" t="n">
-        <v>222581.45</v>
+        <v>217206.554642013</v>
       </c>
       <c r="CD106" t="n">
-        <v>57418.54999999999</v>
+        <v>62793.44535798696</v>
       </c>
       <c r="CE106" t="n">
-        <v>57418.54999999999</v>
+        <v>62793.44535798696</v>
       </c>
       <c r="CF106" t="n">
-        <v>20.506625</v>
+        <v>22.42623048499534</v>
       </c>
     </row>
     <row r="107">
@@ -34944,16 +34944,16 @@
         <v>120000</v>
       </c>
       <c r="CC107" t="n">
-        <v>114777.54</v>
+        <v>113882.6550397313</v>
       </c>
       <c r="CD107" t="n">
-        <v>5222.460000000006</v>
+        <v>6117.344960268718</v>
       </c>
       <c r="CE107" t="n">
-        <v>5222.460000000006</v>
+        <v>6117.344960268718</v>
       </c>
       <c r="CF107" t="n">
-        <v>4.352050000000006</v>
+        <v>5.097787466890598</v>
       </c>
     </row>
     <row r="108">
@@ -35264,16 +35264,16 @@
         <v>141000</v>
       </c>
       <c r="CC108" t="n">
-        <v>105621.5</v>
+        <v>106814.0979141332</v>
       </c>
       <c r="CD108" t="n">
-        <v>35378.5</v>
+        <v>34185.90208586676</v>
       </c>
       <c r="CE108" t="n">
-        <v>35378.5</v>
+        <v>34185.90208586676</v>
       </c>
       <c r="CF108" t="n">
-        <v>25.09113475177305</v>
+        <v>24.2453206282743</v>
       </c>
     </row>
     <row r="109">
@@ -35564,16 +35564,16 @@
         <v>160000</v>
       </c>
       <c r="CC109" t="n">
-        <v>136442.82</v>
+        <v>137237.0639330772</v>
       </c>
       <c r="CD109" t="n">
-        <v>23557.17999999999</v>
+        <v>22762.93606692276</v>
       </c>
       <c r="CE109" t="n">
-        <v>23557.17999999999</v>
+        <v>22762.93606692276</v>
       </c>
       <c r="CF109" t="n">
-        <v>14.72323749999999</v>
+        <v>14.22683504182672</v>
       </c>
     </row>
     <row r="110">
@@ -35864,16 +35864,16 @@
         <v>84900</v>
       </c>
       <c r="CC110" t="n">
-        <v>103169</v>
+        <v>105582.8923750045</v>
       </c>
       <c r="CD110" t="n">
-        <v>-18269</v>
+        <v>-20682.89237500449</v>
       </c>
       <c r="CE110" t="n">
-        <v>18269</v>
+        <v>20682.89237500449</v>
       </c>
       <c r="CF110" t="n">
-        <v>21.51825677267373</v>
+        <v>24.36147511779092</v>
       </c>
     </row>
     <row r="111">
@@ -36188,16 +36188,16 @@
         <v>395000</v>
       </c>
       <c r="CC111" t="n">
-        <v>303820.13</v>
+        <v>302986.8140185743</v>
       </c>
       <c r="CD111" t="n">
-        <v>91179.87</v>
+        <v>92013.18598142575</v>
       </c>
       <c r="CE111" t="n">
-        <v>91179.87</v>
+        <v>92013.18598142575</v>
       </c>
       <c r="CF111" t="n">
-        <v>23.08351139240506</v>
+        <v>23.29447746365209</v>
       </c>
     </row>
     <row r="112">
@@ -36512,16 +36512,16 @@
         <v>260000</v>
       </c>
       <c r="CC112" t="n">
-        <v>239658.31</v>
+        <v>239817.8008223223</v>
       </c>
       <c r="CD112" t="n">
-        <v>20341.69</v>
+        <v>20182.19917767774</v>
       </c>
       <c r="CE112" t="n">
-        <v>20341.69</v>
+        <v>20182.19917767774</v>
       </c>
       <c r="CF112" t="n">
-        <v>7.823726923076924</v>
+        <v>7.762384299106824</v>
       </c>
     </row>
     <row r="113">
@@ -36836,16 +36836,16 @@
         <v>293077</v>
       </c>
       <c r="CC113" t="n">
-        <v>306472.56</v>
+        <v>305803.6036875761</v>
       </c>
       <c r="CD113" t="n">
-        <v>-13395.56</v>
+        <v>-12726.60368757608</v>
       </c>
       <c r="CE113" t="n">
-        <v>13395.56</v>
+        <v>12726.60368757608</v>
       </c>
       <c r="CF113" t="n">
-        <v>4.570662317411464</v>
+        <v>4.342409567306911</v>
       </c>
     </row>
     <row r="114">
@@ -37164,16 +37164,16 @@
         <v>238000</v>
       </c>
       <c r="CC114" t="n">
-        <v>270615.66</v>
+        <v>270829.4428880178</v>
       </c>
       <c r="CD114" t="n">
-        <v>-32615.65999999997</v>
+        <v>-32829.4428880178</v>
       </c>
       <c r="CE114" t="n">
-        <v>32615.65999999997</v>
+        <v>32829.4428880178</v>
       </c>
       <c r="CF114" t="n">
-        <v>13.7040588235294</v>
+        <v>13.79388356639403</v>
       </c>
     </row>
     <row r="115">
@@ -37482,16 +37482,16 @@
         <v>230000</v>
       </c>
       <c r="CC115" t="n">
-        <v>235996.85</v>
+        <v>231982.3015313199</v>
       </c>
       <c r="CD115" t="n">
-        <v>-5996.850000000006</v>
+        <v>-1982.301531319885</v>
       </c>
       <c r="CE115" t="n">
-        <v>5996.850000000006</v>
+        <v>1982.301531319885</v>
       </c>
       <c r="CF115" t="n">
-        <v>2.607326086956524</v>
+        <v>0.8618702310086456</v>
       </c>
     </row>
     <row r="116">
@@ -37806,16 +37806,16 @@
         <v>317000</v>
       </c>
       <c r="CC116" t="n">
-        <v>309364.14</v>
+        <v>308832.2082841732</v>
       </c>
       <c r="CD116" t="n">
-        <v>7635.859999999986</v>
+        <v>8167.791715826781</v>
       </c>
       <c r="CE116" t="n">
-        <v>7635.859999999986</v>
+        <v>8167.791715826781</v>
       </c>
       <c r="CF116" t="n">
-        <v>2.408788643533119</v>
+        <v>2.576590446633054</v>
       </c>
     </row>
     <row r="117">
@@ -38130,16 +38130,16 @@
         <v>337500</v>
       </c>
       <c r="CC117" t="n">
-        <v>333308.04</v>
+        <v>336711.7897728881</v>
       </c>
       <c r="CD117" t="n">
-        <v>4191.960000000021</v>
+        <v>788.2102271118783</v>
       </c>
       <c r="CE117" t="n">
-        <v>4191.960000000021</v>
+        <v>788.2102271118783</v>
       </c>
       <c r="CF117" t="n">
-        <v>1.242062222222228</v>
+        <v>0.2335437709961121</v>
       </c>
     </row>
     <row r="118">
@@ -38450,16 +38450,16 @@
         <v>144000</v>
       </c>
       <c r="CC118" t="n">
-        <v>140591.75</v>
+        <v>142939.9648215331</v>
       </c>
       <c r="CD118" t="n">
-        <v>3408.25</v>
+        <v>1060.035178466933</v>
       </c>
       <c r="CE118" t="n">
-        <v>3408.25</v>
+        <v>1060.035178466933</v>
       </c>
       <c r="CF118" t="n">
-        <v>2.366840277777778</v>
+        <v>0.7361355406020367</v>
       </c>
     </row>
     <row r="119">
@@ -38756,16 +38756,16 @@
         <v>84500</v>
       </c>
       <c r="CC119" t="n">
-        <v>84713</v>
+        <v>85129.83820158374</v>
       </c>
       <c r="CD119" t="n">
-        <v>-213</v>
+        <v>-629.8382015837415</v>
       </c>
       <c r="CE119" t="n">
-        <v>213</v>
+        <v>629.8382015837415</v>
       </c>
       <c r="CF119" t="n">
-        <v>0.2520710059171598</v>
+        <v>0.7453706527618242</v>
       </c>
     </row>
     <row r="120">
@@ -39074,16 +39074,16 @@
         <v>134900</v>
       </c>
       <c r="CC120" t="n">
-        <v>137353.63</v>
+        <v>136257.642836919</v>
       </c>
       <c r="CD120" t="n">
-        <v>-2453.630000000005</v>
+        <v>-1357.642836919025</v>
       </c>
       <c r="CE120" t="n">
-        <v>2453.630000000005</v>
+        <v>1357.642836919025</v>
       </c>
       <c r="CF120" t="n">
-        <v>1.818851000741293</v>
+        <v>1.006406847234266</v>
       </c>
     </row>
     <row r="121">
@@ -39398,16 +39398,16 @@
         <v>283463</v>
       </c>
       <c r="CC121" t="n">
-        <v>286168.46</v>
+        <v>280085.2064456089</v>
       </c>
       <c r="CD121" t="n">
-        <v>-2705.460000000021</v>
+        <v>3377.79355439113</v>
       </c>
       <c r="CE121" t="n">
-        <v>2705.460000000021</v>
+        <v>3377.79355439113</v>
       </c>
       <c r="CF121" t="n">
-        <v>0.9544314425515926</v>
+        <v>1.191617090904679</v>
       </c>
     </row>
     <row r="122">
@@ -39726,16 +39726,16 @@
         <v>175500</v>
       </c>
       <c r="CC122" t="n">
-        <v>178241.72</v>
+        <v>176974.6231653522</v>
       </c>
       <c r="CD122" t="n">
-        <v>-2741.720000000001</v>
+        <v>-1474.623165352183</v>
       </c>
       <c r="CE122" t="n">
-        <v>2741.720000000001</v>
+        <v>1474.623165352183</v>
       </c>
       <c r="CF122" t="n">
-        <v>1.562233618233619</v>
+        <v>0.8402411198587936</v>
       </c>
     </row>
     <row r="123">
@@ -40048,16 +40048,16 @@
         <v>181000</v>
       </c>
       <c r="CC123" t="n">
-        <v>179603.72</v>
+        <v>179472.5435363131</v>
       </c>
       <c r="CD123" t="n">
-        <v>1396.279999999999</v>
+        <v>1527.456463686889</v>
       </c>
       <c r="CE123" t="n">
-        <v>1396.279999999999</v>
+        <v>1527.456463686889</v>
       </c>
       <c r="CF123" t="n">
-        <v>0.7714254143646402</v>
+        <v>0.8438985987220381</v>
       </c>
     </row>
     <row r="124">
@@ -40368,16 +40368,16 @@
         <v>108959</v>
       </c>
       <c r="CC124" t="n">
-        <v>130529.82</v>
+        <v>134943.0639196365</v>
       </c>
       <c r="CD124" t="n">
-        <v>-21570.82000000001</v>
+        <v>-25984.06391963645</v>
       </c>
       <c r="CE124" t="n">
-        <v>21570.82000000001</v>
+        <v>25984.06391963645</v>
       </c>
       <c r="CF124" t="n">
-        <v>19.79718976862857</v>
+        <v>23.84756093543117</v>
       </c>
     </row>
     <row r="125">
@@ -40700,16 +40700,16 @@
         <v>114500</v>
       </c>
       <c r="CC125" t="n">
-        <v>120388</v>
+        <v>121522.5420104805</v>
       </c>
       <c r="CD125" t="n">
-        <v>-5888</v>
+        <v>-7022.542010480538</v>
       </c>
       <c r="CE125" t="n">
-        <v>5888</v>
+        <v>7022.542010480538</v>
       </c>
       <c r="CF125" t="n">
-        <v>5.14235807860262</v>
+        <v>6.13322446330178</v>
       </c>
     </row>
     <row r="126">
@@ -41024,16 +41024,16 @@
         <v>402000</v>
       </c>
       <c r="CC126" t="n">
-        <v>328544.71</v>
+        <v>342144.512746278</v>
       </c>
       <c r="CD126" t="n">
-        <v>73455.28999999998</v>
+        <v>59855.48725372204</v>
       </c>
       <c r="CE126" t="n">
-        <v>73455.28999999998</v>
+        <v>59855.48725372204</v>
       </c>
       <c r="CF126" t="n">
-        <v>18.27246019900497</v>
+        <v>14.88942468998061</v>
       </c>
     </row>
     <row r="127">
@@ -41344,16 +41344,16 @@
         <v>245350</v>
       </c>
       <c r="CC127" t="n">
-        <v>251302.88</v>
+        <v>248707.4195414178</v>
       </c>
       <c r="CD127" t="n">
-        <v>-5952.880000000005</v>
+        <v>-3357.419541417767</v>
       </c>
       <c r="CE127" t="n">
-        <v>5952.880000000005</v>
+        <v>3357.419541417767</v>
       </c>
       <c r="CF127" t="n">
-        <v>2.426280823313635</v>
+        <v>1.368420436689532</v>
       </c>
     </row>
     <row r="128">
@@ -41668,16 +41668,16 @@
         <v>194201</v>
       </c>
       <c r="CC128" t="n">
-        <v>191638.58</v>
+        <v>189270.3639292398</v>
       </c>
       <c r="CD128" t="n">
-        <v>2562.420000000013</v>
+        <v>4930.636070760229</v>
       </c>
       <c r="CE128" t="n">
-        <v>2562.420000000013</v>
+        <v>4930.636070760229</v>
       </c>
       <c r="CF128" t="n">
-        <v>1.319467973903333</v>
+        <v>2.538934439452026</v>
       </c>
     </row>
     <row r="129">
@@ -41996,16 +41996,16 @@
         <v>140000</v>
       </c>
       <c r="CC129" t="n">
-        <v>144315.23</v>
+        <v>143317.5128325794</v>
       </c>
       <c r="CD129" t="n">
-        <v>-4315.23000000001</v>
+        <v>-3317.512832579378</v>
       </c>
       <c r="CE129" t="n">
-        <v>4315.23000000001</v>
+        <v>3317.512832579378</v>
       </c>
       <c r="CF129" t="n">
-        <v>3.08230714285715</v>
+        <v>2.369652023270984</v>
       </c>
     </row>
     <row r="130">
@@ -42318,16 +42318,16 @@
         <v>205000</v>
       </c>
       <c r="CC130" t="n">
-        <v>197775.1</v>
+        <v>197772.6499739697</v>
       </c>
       <c r="CD130" t="n">
-        <v>7224.899999999994</v>
+        <v>7227.350026030326</v>
       </c>
       <c r="CE130" t="n">
-        <v>7224.899999999994</v>
+        <v>7227.350026030326</v>
       </c>
       <c r="CF130" t="n">
-        <v>3.524341463414631</v>
+        <v>3.525536598063574</v>
       </c>
     </row>
     <row r="131">
@@ -42620,16 +42620,16 @@
         <v>113000</v>
       </c>
       <c r="CC131" t="n">
-        <v>114541.08</v>
+        <v>114700.7852736936</v>
       </c>
       <c r="CD131" t="n">
-        <v>-1541.080000000002</v>
+        <v>-1700.785273693633</v>
       </c>
       <c r="CE131" t="n">
-        <v>1541.080000000002</v>
+        <v>1700.785273693633</v>
       </c>
       <c r="CF131" t="n">
-        <v>1.363787610619471</v>
+        <v>1.505119711233303</v>
       </c>
     </row>
     <row r="132">
@@ -42940,16 +42940,16 @@
         <v>195400</v>
       </c>
       <c r="CC132" t="n">
-        <v>194503.12</v>
+        <v>192387.7176549555</v>
       </c>
       <c r="CD132" t="n">
-        <v>896.8800000000047</v>
+        <v>3012.282345044514</v>
       </c>
       <c r="CE132" t="n">
-        <v>896.8800000000047</v>
+        <v>3012.282345044514</v>
       </c>
       <c r="CF132" t="n">
-        <v>0.4589969293756421</v>
+        <v>1.541597924792484</v>
       </c>
     </row>
     <row r="133">
@@ -43264,16 +43264,16 @@
         <v>139000</v>
       </c>
       <c r="CC133" t="n">
-        <v>142905.5</v>
+        <v>141834.2584050352</v>
       </c>
       <c r="CD133" t="n">
-        <v>-3905.5</v>
+        <v>-2834.258405035187</v>
       </c>
       <c r="CE133" t="n">
-        <v>3905.5</v>
+        <v>2834.258405035187</v>
       </c>
       <c r="CF133" t="n">
-        <v>2.809712230215827</v>
+        <v>2.039034823766321</v>
       </c>
     </row>
     <row r="134">
@@ -43570,16 +43570,16 @@
         <v>128950</v>
       </c>
       <c r="CC134" t="n">
-        <v>122761</v>
+        <v>123420.3376440937</v>
       </c>
       <c r="CD134" t="n">
-        <v>6189</v>
+        <v>5529.662355906286</v>
       </c>
       <c r="CE134" t="n">
-        <v>6189</v>
+        <v>5529.662355906286</v>
       </c>
       <c r="CF134" t="n">
-        <v>4.7995347033734</v>
+        <v>4.288222067395337</v>
       </c>
     </row>
     <row r="135">
@@ -43898,16 +43898,16 @@
         <v>175000</v>
       </c>
       <c r="CC135" t="n">
-        <v>150628.63</v>
+        <v>152731.7521408366</v>
       </c>
       <c r="CD135" t="n">
-        <v>24371.37</v>
+        <v>22268.24785916338</v>
       </c>
       <c r="CE135" t="n">
-        <v>24371.37</v>
+        <v>22268.24785916338</v>
       </c>
       <c r="CF135" t="n">
-        <v>13.92649714285714</v>
+        <v>12.72471306237908</v>
       </c>
     </row>
     <row r="136">
@@ -44216,16 +44216,16 @@
         <v>128500</v>
       </c>
       <c r="CC136" t="n">
-        <v>132642.5</v>
+        <v>134943.8759929626</v>
       </c>
       <c r="CD136" t="n">
-        <v>-4142.5</v>
+        <v>-6443.875992962596</v>
       </c>
       <c r="CE136" t="n">
-        <v>4142.5</v>
+        <v>6443.875992962596</v>
       </c>
       <c r="CF136" t="n">
-        <v>3.223735408560311</v>
+        <v>5.014689488686845</v>
       </c>
     </row>
     <row r="137">
@@ -44538,16 +44538,16 @@
         <v>160000</v>
       </c>
       <c r="CC137" t="n">
-        <v>172321.5</v>
+        <v>173151.769743946</v>
       </c>
       <c r="CD137" t="n">
-        <v>-12321.5</v>
+        <v>-13151.76974394597</v>
       </c>
       <c r="CE137" t="n">
-        <v>12321.5</v>
+        <v>13151.76974394597</v>
       </c>
       <c r="CF137" t="n">
-        <v>7.7009375</v>
+        <v>8.219856089966234</v>
       </c>
     </row>
     <row r="138">
@@ -44862,16 +44862,16 @@
         <v>170000</v>
       </c>
       <c r="CC138" t="n">
-        <v>168195.85</v>
+        <v>171114.6278848189</v>
       </c>
       <c r="CD138" t="n">
-        <v>1804.149999999994</v>
+        <v>-1114.62788481891</v>
       </c>
       <c r="CE138" t="n">
-        <v>1804.149999999994</v>
+        <v>1114.62788481891</v>
       </c>
       <c r="CF138" t="n">
-        <v>1.06126470588235</v>
+        <v>0.6556634616581826</v>
       </c>
     </row>
     <row r="139">
@@ -45182,16 +45182,16 @@
         <v>176000</v>
       </c>
       <c r="CC139" t="n">
-        <v>169705.27</v>
+        <v>172652.8163616942</v>
       </c>
       <c r="CD139" t="n">
-        <v>6294.73000000001</v>
+        <v>3347.183638305782</v>
       </c>
       <c r="CE139" t="n">
-        <v>6294.73000000001</v>
+        <v>3347.183638305782</v>
       </c>
       <c r="CF139" t="n">
-        <v>3.576551136363642</v>
+        <v>1.901808885401012</v>
       </c>
     </row>
     <row r="140">
@@ -45510,16 +45510,16 @@
         <v>159950</v>
       </c>
       <c r="CC140" t="n">
-        <v>151981.33</v>
+        <v>148101.3905610136</v>
       </c>
       <c r="CD140" t="n">
-        <v>7968.670000000013</v>
+        <v>11848.60943898643</v>
       </c>
       <c r="CE140" t="n">
-        <v>7968.670000000013</v>
+        <v>11848.60943898643</v>
       </c>
       <c r="CF140" t="n">
-        <v>4.981975617380439</v>
+        <v>7.407695804305364</v>
       </c>
     </row>
     <row r="141">
@@ -45834,16 +45834,16 @@
         <v>325000</v>
       </c>
       <c r="CC141" t="n">
-        <v>336197.63</v>
+        <v>328086.1054372294</v>
       </c>
       <c r="CD141" t="n">
-        <v>-11197.63</v>
+        <v>-3086.105437229387</v>
       </c>
       <c r="CE141" t="n">
-        <v>11197.63</v>
+        <v>3086.105437229387</v>
       </c>
       <c r="CF141" t="n">
-        <v>3.445424615384617</v>
+        <v>0.9495709037628884</v>
       </c>
     </row>
     <row r="142">
@@ -46156,16 +46156,16 @@
         <v>180000</v>
       </c>
       <c r="CC142" t="n">
-        <v>168321.55</v>
+        <v>171213.2486676502</v>
       </c>
       <c r="CD142" t="n">
-        <v>11678.45000000001</v>
+        <v>8786.751332349813</v>
       </c>
       <c r="CE142" t="n">
-        <v>11678.45000000001</v>
+        <v>8786.751332349813</v>
       </c>
       <c r="CF142" t="n">
-        <v>6.488027777777784</v>
+        <v>4.881528517972118</v>
       </c>
     </row>
     <row r="143">
@@ -46480,16 +46480,16 @@
         <v>175000</v>
       </c>
       <c r="CC143" t="n">
-        <v>184277.6</v>
+        <v>181938.364778145</v>
       </c>
       <c r="CD143" t="n">
-        <v>-9277.600000000006</v>
+        <v>-6938.364778145042</v>
       </c>
       <c r="CE143" t="n">
-        <v>9277.600000000006</v>
+        <v>6938.364778145042</v>
       </c>
       <c r="CF143" t="n">
-        <v>5.301485714285717</v>
+        <v>3.964779873225738</v>
       </c>
     </row>
     <row r="144">
@@ -46808,16 +46808,16 @@
         <v>144000</v>
       </c>
       <c r="CC144" t="n">
-        <v>145943.3</v>
+        <v>147078.245535865</v>
       </c>
       <c r="CD144" t="n">
-        <v>-1943.299999999988</v>
+        <v>-3078.245535865048</v>
       </c>
       <c r="CE144" t="n">
-        <v>1943.299999999988</v>
+        <v>3078.245535865048</v>
       </c>
       <c r="CF144" t="n">
-        <v>1.349513888888881</v>
+        <v>2.137670511017394</v>
       </c>
     </row>
     <row r="145">
@@ -47132,16 +47132,16 @@
         <v>253293</v>
       </c>
       <c r="CC145" t="n">
-        <v>359284.69</v>
+        <v>369108.246689484</v>
       </c>
       <c r="CD145" t="n">
-        <v>-105991.69</v>
+        <v>-115815.246689484</v>
       </c>
       <c r="CE145" t="n">
-        <v>105991.69</v>
+        <v>115815.246689484</v>
       </c>
       <c r="CF145" t="n">
-        <v>41.84548724204775</v>
+        <v>45.72382446000641</v>
       </c>
     </row>
     <row r="146">
@@ -47456,16 +47456,16 @@
         <v>143000</v>
       </c>
       <c r="CC146" t="n">
-        <v>141047</v>
+        <v>141773.3319339378</v>
       </c>
       <c r="CD146" t="n">
-        <v>1953</v>
+        <v>1226.668066062208</v>
       </c>
       <c r="CE146" t="n">
-        <v>1953</v>
+        <v>1226.668066062208</v>
       </c>
       <c r="CF146" t="n">
-        <v>1.365734265734266</v>
+        <v>0.8578098364071384</v>
       </c>
     </row>
     <row r="147">
@@ -47776,16 +47776,16 @@
         <v>122500</v>
       </c>
       <c r="CC147" t="n">
-        <v>128081.53</v>
+        <v>129354.1252766302</v>
       </c>
       <c r="CD147" t="n">
-        <v>-5581.529999999999</v>
+        <v>-6854.125276630162</v>
       </c>
       <c r="CE147" t="n">
-        <v>5581.529999999999</v>
+        <v>6854.125276630162</v>
       </c>
       <c r="CF147" t="n">
-        <v>4.556351020408163</v>
+        <v>5.595204307453193</v>
       </c>
     </row>
     <row r="148">
@@ -48100,16 +48100,16 @@
         <v>125000</v>
       </c>
       <c r="CC148" t="n">
-        <v>119772.5</v>
+        <v>120687.7731187333</v>
       </c>
       <c r="CD148" t="n">
-        <v>5227.5</v>
+        <v>4312.226881266659</v>
       </c>
       <c r="CE148" t="n">
-        <v>5227.5</v>
+        <v>4312.226881266659</v>
       </c>
       <c r="CF148" t="n">
-        <v>4.182</v>
+        <v>3.449781505013327</v>
       </c>
     </row>
     <row r="149">
@@ -48424,16 +48424,16 @@
         <v>240000</v>
       </c>
       <c r="CC149" t="n">
-        <v>276547.71</v>
+        <v>269741.2639447967</v>
       </c>
       <c r="CD149" t="n">
-        <v>-36547.71000000002</v>
+        <v>-29741.26394479669</v>
       </c>
       <c r="CE149" t="n">
-        <v>36547.71000000002</v>
+        <v>29741.26394479669</v>
       </c>
       <c r="CF149" t="n">
-        <v>15.22821250000001</v>
+        <v>12.39219331033196</v>
       </c>
     </row>
     <row r="150">
@@ -48748,16 +48748,16 @@
         <v>156500</v>
       </c>
       <c r="CC150" t="n">
-        <v>165576</v>
+        <v>164622.9991822966</v>
       </c>
       <c r="CD150" t="n">
-        <v>-9076</v>
+        <v>-8122.999182296597</v>
       </c>
       <c r="CE150" t="n">
-        <v>9076</v>
+        <v>8122.999182296597</v>
       </c>
       <c r="CF150" t="n">
-        <v>5.799361022364217</v>
+        <v>5.190414812969071</v>
       </c>
     </row>
     <row r="151">
@@ -49070,16 +49070,16 @@
         <v>287000</v>
       </c>
       <c r="CC151" t="n">
-        <v>334155.27</v>
+        <v>340917.5935352216</v>
       </c>
       <c r="CD151" t="n">
-        <v>-47155.27000000002</v>
+        <v>-53917.59353522165</v>
       </c>
       <c r="CE151" t="n">
-        <v>47155.27000000002</v>
+        <v>53917.59353522165</v>
       </c>
       <c r="CF151" t="n">
-        <v>16.43040766550524</v>
+        <v>18.78661795652322</v>
       </c>
     </row>
     <row r="152">
@@ -49394,16 +49394,16 @@
         <v>325000</v>
       </c>
       <c r="CC152" t="n">
-        <v>317255.62</v>
+        <v>318747.9912596141</v>
       </c>
       <c r="CD152" t="n">
-        <v>7744.380000000005</v>
+        <v>6252.008740385936</v>
       </c>
       <c r="CE152" t="n">
-        <v>7744.380000000005</v>
+        <v>6252.008740385936</v>
       </c>
       <c r="CF152" t="n">
-        <v>2.382886153846155</v>
+        <v>1.923694997041827</v>
       </c>
     </row>
     <row r="153">
@@ -49718,16 +49718,16 @@
         <v>207500</v>
       </c>
       <c r="CC153" t="n">
-        <v>207842.83</v>
+        <v>204816.745730935</v>
       </c>
       <c r="CD153" t="n">
-        <v>-342.8299999999872</v>
+        <v>2683.254269064957</v>
       </c>
       <c r="CE153" t="n">
-        <v>342.8299999999872</v>
+        <v>2683.254269064957</v>
       </c>
       <c r="CF153" t="n">
-        <v>0.1652192771084276</v>
+        <v>1.293134587501184</v>
       </c>
     </row>
     <row r="154">
@@ -50042,16 +50042,16 @@
         <v>144000</v>
       </c>
       <c r="CC154" t="n">
-        <v>142397.42</v>
+        <v>143256.1127786536</v>
       </c>
       <c r="CD154" t="n">
-        <v>1602.579999999987</v>
+        <v>743.8872213463765</v>
       </c>
       <c r="CE154" t="n">
-        <v>1602.579999999987</v>
+        <v>743.8872213463765</v>
       </c>
       <c r="CF154" t="n">
-        <v>1.112902777777769</v>
+        <v>0.5165883481572059</v>
       </c>
     </row>
     <row r="155">
@@ -50362,16 +50362,16 @@
         <v>118000</v>
       </c>
       <c r="CC155" t="n">
-        <v>100681</v>
+        <v>103667.574270898</v>
       </c>
       <c r="CD155" t="n">
-        <v>17319</v>
+        <v>14332.42572910197</v>
       </c>
       <c r="CE155" t="n">
-        <v>17319</v>
+        <v>14332.42572910197</v>
       </c>
       <c r="CF155" t="n">
-        <v>14.6771186440678</v>
+        <v>12.14612349923896</v>
       </c>
     </row>
     <row r="156">
@@ -50682,16 +50682,16 @@
         <v>135500</v>
       </c>
       <c r="CC156" t="n">
-        <v>124538</v>
+        <v>127574.4734020303</v>
       </c>
       <c r="CD156" t="n">
-        <v>10962</v>
+        <v>7925.526597969743</v>
       </c>
       <c r="CE156" t="n">
-        <v>10962</v>
+        <v>7925.526597969743</v>
       </c>
       <c r="CF156" t="n">
-        <v>8.090036900369004</v>
+        <v>5.849097120272873</v>
       </c>
     </row>
     <row r="157">
@@ -51006,16 +51006,16 @@
         <v>255000</v>
       </c>
       <c r="CC157" t="n">
-        <v>251525.18</v>
+        <v>251304.1007080083</v>
       </c>
       <c r="CD157" t="n">
-        <v>3474.820000000007</v>
+        <v>3695.899291991664</v>
       </c>
       <c r="CE157" t="n">
-        <v>3474.820000000007</v>
+        <v>3695.899291991664</v>
       </c>
       <c r="CF157" t="n">
-        <v>1.362674509803924</v>
+        <v>1.44937227136928</v>
       </c>
     </row>
     <row r="158">
@@ -51328,16 +51328,16 @@
         <v>275000</v>
       </c>
       <c r="CC158" t="n">
-        <v>227731.82</v>
+        <v>227589.9559035241</v>
       </c>
       <c r="CD158" t="n">
-        <v>47268.17999999999</v>
+        <v>47410.0440964759</v>
       </c>
       <c r="CE158" t="n">
-        <v>47268.17999999999</v>
+        <v>47410.0440964759</v>
       </c>
       <c r="CF158" t="n">
-        <v>17.18842909090909</v>
+        <v>17.24001603508215</v>
       </c>
     </row>
     <row r="159">
@@ -51660,16 +51660,16 @@
         <v>181000</v>
       </c>
       <c r="CC159" t="n">
-        <v>160945.82</v>
+        <v>161240.9955884673</v>
       </c>
       <c r="CD159" t="n">
-        <v>20054.17999999999</v>
+        <v>19759.00441153275</v>
       </c>
       <c r="CE159" t="n">
-        <v>20054.17999999999</v>
+        <v>19759.00441153275</v>
       </c>
       <c r="CF159" t="n">
-        <v>11.07965745856353</v>
+        <v>10.91657702294627</v>
       </c>
     </row>
     <row r="160">
@@ -51984,16 +51984,16 @@
         <v>152000</v>
       </c>
       <c r="CC160" t="n">
-        <v>162104.53</v>
+        <v>165358.2900368426</v>
       </c>
       <c r="CD160" t="n">
-        <v>-10104.53</v>
+        <v>-13358.29003684258</v>
       </c>
       <c r="CE160" t="n">
-        <v>10104.53</v>
+        <v>13358.29003684258</v>
       </c>
       <c r="CF160" t="n">
-        <v>6.647717105263157</v>
+        <v>8.788348708449064</v>
       </c>
     </row>
     <row r="161">
@@ -52298,16 +52298,16 @@
         <v>182000</v>
       </c>
       <c r="CC161" t="n">
-        <v>209565.78</v>
+        <v>208234.8754219744</v>
       </c>
       <c r="CD161" t="n">
-        <v>-27565.78</v>
+        <v>-26234.87542197437</v>
       </c>
       <c r="CE161" t="n">
-        <v>27565.78</v>
+        <v>26234.87542197437</v>
       </c>
       <c r="CF161" t="n">
-        <v>15.14603296703297</v>
+        <v>14.41476671537053</v>
       </c>
     </row>
     <row r="162">
@@ -52620,16 +52620,16 @@
         <v>115000</v>
       </c>
       <c r="CC162" t="n">
-        <v>120425.87</v>
+        <v>119611.7182221842</v>
       </c>
       <c r="CD162" t="n">
-        <v>-5425.869999999995</v>
+        <v>-4611.71822218415</v>
       </c>
       <c r="CE162" t="n">
-        <v>5425.869999999995</v>
+        <v>4611.71822218415</v>
       </c>
       <c r="CF162" t="n">
-        <v>4.718147826086953</v>
+        <v>4.010189758421</v>
       </c>
     </row>
     <row r="163">
@@ -52944,16 +52944,16 @@
         <v>310000</v>
       </c>
       <c r="CC163" t="n">
-        <v>327040.53</v>
+        <v>331028.7437061768</v>
       </c>
       <c r="CD163" t="n">
-        <v>-17040.53000000003</v>
+        <v>-21028.74370617676</v>
       </c>
       <c r="CE163" t="n">
-        <v>17040.53000000003</v>
+        <v>21028.74370617676</v>
       </c>
       <c r="CF163" t="n">
-        <v>5.496945161290332</v>
+        <v>6.783465711669921</v>
       </c>
     </row>
     <row r="164">
@@ -53268,16 +53268,16 @@
         <v>311872</v>
       </c>
       <c r="CC164" t="n">
-        <v>261282.2</v>
+        <v>261740.6531236213</v>
       </c>
       <c r="CD164" t="n">
-        <v>50589.79999999999</v>
+        <v>50131.34687637867</v>
       </c>
       <c r="CE164" t="n">
-        <v>50589.79999999999</v>
+        <v>50131.34687637867</v>
       </c>
       <c r="CF164" t="n">
-        <v>16.22133439359737</v>
+        <v>16.07433398201142</v>
       </c>
     </row>
     <row r="165">
@@ -53592,16 +53592,16 @@
         <v>242000</v>
       </c>
       <c r="CC165" t="n">
-        <v>248452.71</v>
+        <v>246690.6256461734</v>
       </c>
       <c r="CD165" t="n">
-        <v>-6452.709999999992</v>
+        <v>-4690.62564617343</v>
       </c>
       <c r="CE165" t="n">
-        <v>6452.709999999992</v>
+        <v>4690.62564617343</v>
       </c>
       <c r="CF165" t="n">
-        <v>2.666409090909088</v>
+        <v>1.938275060402244</v>
       </c>
     </row>
     <row r="166">
@@ -53912,16 +53912,16 @@
         <v>214000</v>
       </c>
       <c r="CC166" t="n">
-        <v>207952.19</v>
+        <v>207382.3745411608</v>
       </c>
       <c r="CD166" t="n">
-        <v>6047.809999999998</v>
+        <v>6617.625458839175</v>
       </c>
       <c r="CE166" t="n">
-        <v>6047.809999999998</v>
+        <v>6617.625458839175</v>
       </c>
       <c r="CF166" t="n">
-        <v>2.826079439252335</v>
+        <v>3.092348345251951</v>
       </c>
     </row>
     <row r="167">
@@ -54236,16 +54236,16 @@
         <v>178900</v>
       </c>
       <c r="CC167" t="n">
-        <v>168454.62</v>
+        <v>172477.9594197027</v>
       </c>
       <c r="CD167" t="n">
-        <v>10445.38</v>
+        <v>6422.040580297296</v>
       </c>
       <c r="CE167" t="n">
-        <v>10445.38</v>
+        <v>6422.040580297296</v>
       </c>
       <c r="CF167" t="n">
-        <v>5.838669647847962</v>
+        <v>3.589737607768193</v>
       </c>
     </row>
     <row r="168">
@@ -54560,16 +54560,16 @@
         <v>155900</v>
       </c>
       <c r="CC168" t="n">
-        <v>139325</v>
+        <v>139913.1405131596</v>
       </c>
       <c r="CD168" t="n">
-        <v>16575</v>
+        <v>15986.85948684037</v>
       </c>
       <c r="CE168" t="n">
-        <v>16575</v>
+        <v>15986.85948684037</v>
       </c>
       <c r="CF168" t="n">
-        <v>10.63181526619628</v>
+        <v>10.25456028661987</v>
       </c>
     </row>
     <row r="169">
@@ -54880,16 +54880,16 @@
         <v>85000</v>
       </c>
       <c r="CC169" t="n">
-        <v>106775.43</v>
+        <v>107930.789110718</v>
       </c>
       <c r="CD169" t="n">
-        <v>-21775.42999999999</v>
+        <v>-22930.78911071805</v>
       </c>
       <c r="CE169" t="n">
-        <v>21775.42999999999</v>
+        <v>22930.78911071805</v>
       </c>
       <c r="CF169" t="n">
-        <v>25.61815294117647</v>
+        <v>26.97739895378594</v>
       </c>
     </row>
     <row r="170">
@@ -55208,16 +55208,16 @@
         <v>239000</v>
       </c>
       <c r="CC170" t="n">
-        <v>200572.68</v>
+        <v>200314.194415539</v>
       </c>
       <c r="CD170" t="n">
-        <v>38427.32000000001</v>
+        <v>38685.80558446099</v>
       </c>
       <c r="CE170" t="n">
-        <v>38427.32000000001</v>
+        <v>38685.80558446099</v>
       </c>
       <c r="CF170" t="n">
-        <v>16.07837656903766</v>
+        <v>16.18652953324728</v>
       </c>
     </row>
     <row r="171">
@@ -55532,16 +55532,16 @@
         <v>149500</v>
       </c>
       <c r="CC171" t="n">
-        <v>178034</v>
+        <v>179406.1473021092</v>
       </c>
       <c r="CD171" t="n">
-        <v>-28534</v>
+        <v>-29906.14730210917</v>
       </c>
       <c r="CE171" t="n">
-        <v>28534</v>
+        <v>29906.14730210917</v>
       </c>
       <c r="CF171" t="n">
-        <v>19.08628762541806</v>
+        <v>20.00411190776533</v>
       </c>
     </row>
     <row r="172">
@@ -55860,16 +55860,16 @@
         <v>62383</v>
       </c>
       <c r="CC172" t="n">
-        <v>124437.5</v>
+        <v>121611.6224540712</v>
       </c>
       <c r="CD172" t="n">
-        <v>-62054.5</v>
+        <v>-59228.62245407123</v>
       </c>
       <c r="CE172" t="n">
-        <v>62054.5</v>
+        <v>59228.62245407123</v>
       </c>
       <c r="CF172" t="n">
-        <v>99.47341423144125</v>
+        <v>94.94353021507659</v>
       </c>
     </row>
     <row r="173">
@@ -56180,16 +56180,16 @@
         <v>35311</v>
       </c>
       <c r="CC173" t="n">
-        <v>82543.5</v>
+        <v>82148.7906139714</v>
       </c>
       <c r="CD173" t="n">
-        <v>-47232.5</v>
+        <v>-46837.7906139714</v>
       </c>
       <c r="CE173" t="n">
-        <v>47232.5</v>
+        <v>46837.7906139714</v>
       </c>
       <c r="CF173" t="n">
-        <v>133.7614341140155</v>
+        <v>132.643625538703</v>
       </c>
     </row>
     <row r="174">
@@ -56500,16 +56500,16 @@
         <v>140000</v>
       </c>
       <c r="CC174" t="n">
-        <v>163696</v>
+        <v>162355.1169197435</v>
       </c>
       <c r="CD174" t="n">
-        <v>-23696</v>
+        <v>-22355.11691974354</v>
       </c>
       <c r="CE174" t="n">
-        <v>23696</v>
+        <v>22355.11691974354</v>
       </c>
       <c r="CF174" t="n">
-        <v>16.92571428571429</v>
+        <v>15.96794065695967</v>
       </c>
     </row>
     <row r="175">
@@ -56822,16 +56822,16 @@
         <v>222500</v>
       </c>
       <c r="CC175" t="n">
-        <v>221936.66</v>
+        <v>221481.2785191206</v>
       </c>
       <c r="CD175" t="n">
-        <v>563.3399999999965</v>
+        <v>1018.721480879438</v>
       </c>
       <c r="CE175" t="n">
-        <v>563.3399999999965</v>
+        <v>1018.721480879438</v>
       </c>
       <c r="CF175" t="n">
-        <v>0.253186516853931</v>
+        <v>0.4578523509570507</v>
       </c>
     </row>
     <row r="176">
@@ -57120,16 +57120,16 @@
         <v>87500</v>
       </c>
       <c r="CC176" t="n">
-        <v>93320</v>
+        <v>93851.72710045947</v>
       </c>
       <c r="CD176" t="n">
-        <v>-5820</v>
+        <v>-6351.727100459466</v>
       </c>
       <c r="CE176" t="n">
-        <v>5820</v>
+        <v>6351.727100459466</v>
       </c>
       <c r="CF176" t="n">
-        <v>6.651428571428572</v>
+        <v>7.259116686239389</v>
       </c>
     </row>
     <row r="177">
@@ -57444,16 +57444,16 @@
         <v>438780</v>
       </c>
       <c r="CC177" t="n">
-        <v>400988.01</v>
+        <v>397782.9401881314</v>
       </c>
       <c r="CD177" t="n">
-        <v>37791.98999999999</v>
+        <v>40997.05981186865</v>
       </c>
       <c r="CE177" t="n">
-        <v>37791.98999999999</v>
+        <v>40997.05981186865</v>
       </c>
       <c r="CF177" t="n">
-        <v>8.612970053329684</v>
+        <v>9.343420350031598</v>
       </c>
     </row>
     <row r="178">
@@ -57766,16 +57766,16 @@
         <v>144500</v>
       </c>
       <c r="CC178" t="n">
-        <v>140117.9</v>
+        <v>140094.9338237934</v>
       </c>
       <c r="CD178" t="n">
-        <v>4382.100000000006</v>
+        <v>4405.066176206572</v>
       </c>
       <c r="CE178" t="n">
-        <v>4382.100000000006</v>
+        <v>4405.066176206572</v>
       </c>
       <c r="CF178" t="n">
-        <v>3.032595155709346</v>
+        <v>3.048488703257143</v>
       </c>
     </row>
     <row r="179">
@@ -58088,16 +58088,16 @@
         <v>248000</v>
       </c>
       <c r="CC179" t="n">
-        <v>223019.2</v>
+        <v>222547.4505121983</v>
       </c>
       <c r="CD179" t="n">
-        <v>24980.79999999999</v>
+        <v>25452.54948780168</v>
       </c>
       <c r="CE179" t="n">
-        <v>24980.79999999999</v>
+        <v>25452.54948780168</v>
       </c>
       <c r="CF179" t="n">
-        <v>10.07290322580645</v>
+        <v>10.26312479346842</v>
       </c>
     </row>
     <row r="180">
@@ -58408,16 +58408,16 @@
         <v>119000</v>
       </c>
       <c r="CC180" t="n">
-        <v>120192.5</v>
+        <v>119506.0748314734</v>
       </c>
       <c r="CD180" t="n">
-        <v>-1192.5</v>
+        <v>-506.0748314733792</v>
       </c>
       <c r="CE180" t="n">
-        <v>1192.5</v>
+        <v>506.0748314733792</v>
       </c>
       <c r="CF180" t="n">
-        <v>1.002100840336134</v>
+        <v>0.4252729676246884</v>
       </c>
     </row>
     <row r="181">
@@ -58732,16 +58732,16 @@
         <v>285000</v>
       </c>
       <c r="CC181" t="n">
-        <v>329557.56</v>
+        <v>328051.7878686152</v>
       </c>
       <c r="CD181" t="n">
-        <v>-44557.56</v>
+        <v>-43051.78786861524</v>
       </c>
       <c r="CE181" t="n">
-        <v>44557.56</v>
+        <v>43051.78786861524</v>
       </c>
       <c r="CF181" t="n">
-        <v>15.63423157894737</v>
+        <v>15.10589048021587</v>
       </c>
     </row>
     <row r="182">
@@ -59052,16 +59052,16 @@
         <v>75000</v>
       </c>
       <c r="CC182" t="n">
-        <v>88645</v>
+        <v>87722.66391788685</v>
       </c>
       <c r="CD182" t="n">
-        <v>-13645</v>
+        <v>-12722.66391788685</v>
       </c>
       <c r="CE182" t="n">
-        <v>13645</v>
+        <v>12722.66391788685</v>
       </c>
       <c r="CF182" t="n">
-        <v>18.19333333333334</v>
+        <v>16.9635518905158</v>
       </c>
     </row>
     <row r="183">
@@ -59372,16 +59372,16 @@
         <v>126175</v>
       </c>
       <c r="CC183" t="n">
-        <v>129611.75</v>
+        <v>127585.6243501098</v>
       </c>
       <c r="CD183" t="n">
-        <v>-3436.75</v>
+        <v>-1410.624350109778</v>
       </c>
       <c r="CE183" t="n">
-        <v>3436.75</v>
+        <v>1410.624350109778</v>
       </c>
       <c r="CF183" t="n">
-        <v>2.723796314642362</v>
+        <v>1.117990370604143</v>
       </c>
     </row>
     <row r="184">
@@ -59696,16 +59696,16 @@
         <v>246578</v>
       </c>
       <c r="CC184" t="n">
-        <v>206248.16</v>
+        <v>207782.5380737244</v>
       </c>
       <c r="CD184" t="n">
-        <v>40329.84</v>
+        <v>38795.4619262756</v>
       </c>
       <c r="CE184" t="n">
-        <v>40329.84</v>
+        <v>38795.4619262756</v>
       </c>
       <c r="CF184" t="n">
-        <v>16.35581438733383</v>
+        <v>15.7335455418876</v>
       </c>
     </row>
     <row r="185">
@@ -60018,16 +60018,16 @@
         <v>244400</v>
       </c>
       <c r="CC185" t="n">
-        <v>230426.55</v>
+        <v>227727.434621669</v>
       </c>
       <c r="CD185" t="n">
-        <v>13973.45000000001</v>
+        <v>16672.56537833103</v>
       </c>
       <c r="CE185" t="n">
-        <v>13973.45000000001</v>
+        <v>16672.56537833103</v>
       </c>
       <c r="CF185" t="n">
-        <v>5.717450900163671</v>
+        <v>6.821835261182908</v>
       </c>
     </row>
     <row r="186">
@@ -60346,16 +60346,16 @@
         <v>107000</v>
       </c>
       <c r="CC186" t="n">
-        <v>145882.97</v>
+        <v>146027.8462579999</v>
       </c>
       <c r="CD186" t="n">
-        <v>-38882.97</v>
+        <v>-39027.84625799989</v>
       </c>
       <c r="CE186" t="n">
-        <v>38882.97</v>
+        <v>39027.84625799989</v>
       </c>
       <c r="CF186" t="n">
-        <v>36.33922429906542</v>
+        <v>36.47462267102794</v>
       </c>
     </row>
     <row r="187">
@@ -60670,16 +60670,16 @@
         <v>451950</v>
       </c>
       <c r="CC187" t="n">
-        <v>365854.51</v>
+        <v>381280.0931723448</v>
       </c>
       <c r="CD187" t="n">
-        <v>86095.48999999999</v>
+        <v>70669.90682765516</v>
       </c>
       <c r="CE187" t="n">
-        <v>86095.48999999999</v>
+        <v>70669.90682765516</v>
       </c>
       <c r="CF187" t="n">
-        <v>19.04978205553711</v>
+        <v>15.63666485842574</v>
       </c>
     </row>
     <row r="188">
@@ -60994,16 +60994,16 @@
         <v>219210</v>
       </c>
       <c r="CC188" t="n">
-        <v>218357.11</v>
+        <v>221170.7061846775</v>
       </c>
       <c r="CD188" t="n">
-        <v>852.890000000014</v>
+        <v>-1960.706184677489</v>
       </c>
       <c r="CE188" t="n">
-        <v>852.890000000014</v>
+        <v>1960.706184677489</v>
       </c>
       <c r="CF188" t="n">
-        <v>0.3890744035399908</v>
+        <v>0.89444194365106</v>
       </c>
     </row>
     <row r="189">
@@ -61314,16 +61314,16 @@
         <v>153575</v>
       </c>
       <c r="CC189" t="n">
-        <v>137017.19</v>
+        <v>136644.4258657865</v>
       </c>
       <c r="CD189" t="n">
-        <v>16557.81</v>
+        <v>16930.57413421347</v>
       </c>
       <c r="CE189" t="n">
-        <v>16557.81</v>
+        <v>16930.57413421347</v>
       </c>
       <c r="CF189" t="n">
-        <v>10.78157903304574</v>
+        <v>11.02430352219663</v>
       </c>
     </row>
     <row r="190">
@@ -61636,16 +61636,16 @@
         <v>145000</v>
       </c>
       <c r="CC190" t="n">
-        <v>140132.36</v>
+        <v>139169.6884533391</v>
       </c>
       <c r="CD190" t="n">
-        <v>4867.640000000014</v>
+        <v>5830.311546660872</v>
       </c>
       <c r="CE190" t="n">
-        <v>4867.640000000014</v>
+        <v>5830.311546660872</v>
       </c>
       <c r="CF190" t="n">
-        <v>3.356993103448286</v>
+        <v>4.020904514938533</v>
       </c>
     </row>
     <row r="191">
@@ -61956,16 +61956,16 @@
         <v>210000</v>
       </c>
       <c r="CC191" t="n">
-        <v>231353.49</v>
+        <v>226631.5040933355</v>
       </c>
       <c r="CD191" t="n">
-        <v>-21353.48999999999</v>
+        <v>-16631.50409333553</v>
       </c>
       <c r="CE191" t="n">
-        <v>21353.48999999999</v>
+        <v>16631.50409333553</v>
       </c>
       <c r="CF191" t="n">
-        <v>10.16832857142857</v>
+        <v>7.919763853969301</v>
       </c>
     </row>
     <row r="192">
@@ -62276,16 +62276,16 @@
         <v>200000</v>
       </c>
       <c r="CC192" t="n">
-        <v>155836.91</v>
+        <v>163549.3928890598</v>
       </c>
       <c r="CD192" t="n">
-        <v>44163.09</v>
+        <v>36450.60711094015</v>
       </c>
       <c r="CE192" t="n">
-        <v>44163.09</v>
+        <v>36450.60711094015</v>
       </c>
       <c r="CF192" t="n">
-        <v>22.081545</v>
+        <v>18.22530355547008</v>
       </c>
     </row>
     <row r="193">
@@ -62596,16 +62596,16 @@
         <v>179900</v>
       </c>
       <c r="CC193" t="n">
-        <v>228029.91</v>
+        <v>225284.718080313</v>
       </c>
       <c r="CD193" t="n">
-        <v>-48129.91</v>
+        <v>-45384.71808031297</v>
       </c>
       <c r="CE193" t="n">
-        <v>48129.91</v>
+        <v>45384.71808031297</v>
       </c>
       <c r="CF193" t="n">
-        <v>26.75370205669817</v>
+        <v>25.22774768221955</v>
       </c>
     </row>
     <row r="194">
@@ -62916,16 +62916,16 @@
         <v>137500</v>
       </c>
       <c r="CC194" t="n">
-        <v>134777.95</v>
+        <v>135932.5678281825</v>
       </c>
       <c r="CD194" t="n">
-        <v>2722.049999999988</v>
+        <v>1567.432171817549</v>
       </c>
       <c r="CE194" t="n">
-        <v>2722.049999999988</v>
+        <v>1567.432171817549</v>
       </c>
       <c r="CF194" t="n">
-        <v>1.979672727272719</v>
+        <v>1.139950670412763</v>
       </c>
     </row>
     <row r="195">
@@ -63236,16 +63236,16 @@
         <v>108480</v>
       </c>
       <c r="CC195" t="n">
-        <v>118254.25</v>
+        <v>118143.0827366259</v>
       </c>
       <c r="CD195" t="n">
-        <v>-9774.25</v>
+        <v>-9663.082736625889</v>
       </c>
       <c r="CE195" t="n">
-        <v>9774.25</v>
+        <v>9663.082736625889</v>
       </c>
       <c r="CF195" t="n">
-        <v>9.010186209439528</v>
+        <v>8.907709012376372</v>
       </c>
     </row>
     <row r="196">
@@ -63560,16 +63560,16 @@
         <v>215000</v>
       </c>
       <c r="CC196" t="n">
-        <v>223933.07</v>
+        <v>224433.7397953002</v>
       </c>
       <c r="CD196" t="n">
-        <v>-8933.070000000007</v>
+        <v>-9433.739795300178</v>
       </c>
       <c r="CE196" t="n">
-        <v>8933.070000000007</v>
+        <v>9433.739795300178</v>
       </c>
       <c r="CF196" t="n">
-        <v>4.154916279069771</v>
+        <v>4.387785951302408</v>
       </c>
     </row>
     <row r="197">
@@ -63884,16 +63884,16 @@
         <v>178000</v>
       </c>
       <c r="CC197" t="n">
-        <v>174476.34</v>
+        <v>176754.1995061489</v>
       </c>
       <c r="CD197" t="n">
-        <v>3523.660000000003</v>
+        <v>1245.800493851071</v>
       </c>
       <c r="CE197" t="n">
-        <v>3523.660000000003</v>
+        <v>1245.800493851071</v>
       </c>
       <c r="CF197" t="n">
-        <v>1.979584269662924</v>
+        <v>0.6998879178938602</v>
       </c>
     </row>
     <row r="198">
@@ -64208,16 +64208,16 @@
         <v>274900</v>
       </c>
       <c r="CC198" t="n">
-        <v>313545.63</v>
+        <v>320497.6409085433</v>
       </c>
       <c r="CD198" t="n">
-        <v>-38645.63</v>
+        <v>-45597.64090854325</v>
       </c>
       <c r="CE198" t="n">
-        <v>38645.63</v>
+        <v>45597.64090854325</v>
       </c>
       <c r="CF198" t="n">
-        <v>14.05806838850491</v>
+        <v>16.58699196382075</v>
       </c>
     </row>
     <row r="199">
@@ -64536,16 +64536,16 @@
         <v>174000</v>
       </c>
       <c r="CC199" t="n">
-        <v>169544.54</v>
+        <v>173174.7565303459</v>
       </c>
       <c r="CD199" t="n">
-        <v>4455.459999999992</v>
+        <v>825.2434696540586</v>
       </c>
       <c r="CE199" t="n">
-        <v>4455.459999999992</v>
+        <v>825.2434696540586</v>
       </c>
       <c r="CF199" t="n">
-        <v>2.560609195402294</v>
+        <v>0.4742778561230221</v>
       </c>
     </row>
     <row r="200">
@@ -64856,16 +64856,16 @@
         <v>119500</v>
       </c>
       <c r="CC200" t="n">
-        <v>111175.84</v>
+        <v>112846.2433660834</v>
       </c>
       <c r="CD200" t="n">
-        <v>8324.160000000003</v>
+        <v>6653.756633916608</v>
       </c>
       <c r="CE200" t="n">
-        <v>8324.160000000003</v>
+        <v>6653.756633916608</v>
       </c>
       <c r="CF200" t="n">
-        <v>6.96582426778243</v>
+        <v>5.567997183193814</v>
       </c>
     </row>
     <row r="201">
@@ -65182,16 +65182,16 @@
         <v>217000</v>
       </c>
       <c r="CC201" t="n">
-        <v>203070.59</v>
+        <v>200920.3847925562</v>
       </c>
       <c r="CD201" t="n">
-        <v>13929.41</v>
+        <v>16079.61520744377</v>
       </c>
       <c r="CE201" t="n">
-        <v>13929.41</v>
+        <v>16079.61520744377</v>
       </c>
       <c r="CF201" t="n">
-        <v>6.419082949308757</v>
+        <v>7.409960925089296</v>
       </c>
     </row>
     <row r="202">
@@ -65488,16 +65488,16 @@
         <v>67000</v>
       </c>
       <c r="CC202" t="n">
-        <v>79593.5</v>
+        <v>76174.49020964465</v>
       </c>
       <c r="CD202" t="n">
-        <v>-12593.5</v>
+        <v>-9174.490209644646</v>
       </c>
       <c r="CE202" t="n">
-        <v>12593.5</v>
+        <v>9174.490209644646</v>
       </c>
       <c r="CF202" t="n">
-        <v>18.79626865671642</v>
+        <v>13.69326896961887</v>
       </c>
     </row>
     <row r="203">
@@ -65808,16 +65808,16 @@
         <v>185900</v>
       </c>
       <c r="CC203" t="n">
-        <v>187748.14</v>
+        <v>188582.2249405172</v>
       </c>
       <c r="CD203" t="n">
-        <v>-1848.140000000014</v>
+        <v>-2682.224940517219</v>
       </c>
       <c r="CE203" t="n">
-        <v>1848.140000000014</v>
+        <v>2682.224940517219</v>
       </c>
       <c r="CF203" t="n">
-        <v>0.9941581495427725</v>
+        <v>1.442832135834975</v>
       </c>
     </row>
     <row r="204">
@@ -66132,16 +66132,16 @@
         <v>155000</v>
       </c>
       <c r="CC204" t="n">
-        <v>142877.3</v>
+        <v>143512.9290727739</v>
       </c>
       <c r="CD204" t="n">
-        <v>12122.70000000001</v>
+        <v>11487.07092722607</v>
       </c>
       <c r="CE204" t="n">
-        <v>12122.70000000001</v>
+        <v>11487.07092722607</v>
       </c>
       <c r="CF204" t="n">
-        <v>7.821096774193556</v>
+        <v>7.411013501436176</v>
       </c>
     </row>
     <row r="205">
@@ -66456,16 +66456,16 @@
         <v>350000</v>
       </c>
       <c r="CC205" t="n">
-        <v>340010.21</v>
+        <v>341789.3073850293</v>
       </c>
       <c r="CD205" t="n">
-        <v>9989.789999999979</v>
+        <v>8210.692614970671</v>
       </c>
       <c r="CE205" t="n">
-        <v>9989.789999999979</v>
+        <v>8210.692614970671</v>
       </c>
       <c r="CF205" t="n">
-        <v>2.854225714285708</v>
+        <v>2.345912175705906</v>
       </c>
     </row>
     <row r="206">
@@ -66784,16 +66784,16 @@
         <v>260000</v>
       </c>
       <c r="CC206" t="n">
-        <v>244847.82</v>
+        <v>243504.5022709229</v>
       </c>
       <c r="CD206" t="n">
-        <v>15152.17999999999</v>
+        <v>16495.49772907712</v>
       </c>
       <c r="CE206" t="n">
-        <v>15152.17999999999</v>
+        <v>16495.49772907712</v>
       </c>
       <c r="CF206" t="n">
-        <v>5.827761538461536</v>
+        <v>6.3444222034912</v>
       </c>
     </row>
     <row r="207">
@@ -67112,16 +67112,16 @@
         <v>130000</v>
       </c>
       <c r="CC207" t="n">
-        <v>124970.97</v>
+        <v>126345.4143220942</v>
       </c>
       <c r="CD207" t="n">
-        <v>5029.029999999999</v>
+        <v>3654.58567790575</v>
       </c>
       <c r="CE207" t="n">
-        <v>5029.029999999999</v>
+        <v>3654.58567790575</v>
       </c>
       <c r="CF207" t="n">
-        <v>3.868484615384614</v>
+        <v>2.811219752235192</v>
       </c>
     </row>
     <row r="208">
@@ -67434,16 +67434,16 @@
         <v>190000</v>
       </c>
       <c r="CC208" t="n">
-        <v>202577.46</v>
+        <v>197763.3056398183</v>
       </c>
       <c r="CD208" t="n">
-        <v>-12577.45999999999</v>
+        <v>-7763.305639818282</v>
       </c>
       <c r="CE208" t="n">
-        <v>12577.45999999999</v>
+        <v>7763.305639818282</v>
       </c>
       <c r="CF208" t="n">
-        <v>6.61971578947368</v>
+        <v>4.085950336746464</v>
       </c>
     </row>
     <row r="209">
@@ -67758,16 +67758,16 @@
         <v>153337</v>
       </c>
       <c r="CC209" t="n">
-        <v>152158.8</v>
+        <v>151904.4816951726</v>
       </c>
       <c r="CD209" t="n">
-        <v>1178.200000000012</v>
+        <v>1432.518304827419</v>
       </c>
       <c r="CE209" t="n">
-        <v>1178.200000000012</v>
+        <v>1432.518304827419</v>
       </c>
       <c r="CF209" t="n">
-        <v>0.7683729302125459</v>
+        <v>0.9342287281135142</v>
       </c>
     </row>
     <row r="210">
@@ -68082,16 +68082,16 @@
         <v>241500</v>
       </c>
       <c r="CC210" t="n">
-        <v>182697.16</v>
+        <v>176295.7344069985</v>
       </c>
       <c r="CD210" t="n">
-        <v>58802.84</v>
+        <v>65204.26559300153</v>
       </c>
       <c r="CE210" t="n">
-        <v>58802.84</v>
+        <v>65204.26559300153</v>
       </c>
       <c r="CF210" t="n">
-        <v>24.34900207039338</v>
+        <v>26.9996958977232</v>
       </c>
     </row>
     <row r="211">
@@ -68404,16 +68404,16 @@
         <v>149000</v>
       </c>
       <c r="CC211" t="n">
-        <v>141816</v>
+        <v>140654.4744987415</v>
       </c>
       <c r="CD211" t="n">
-        <v>7184</v>
+        <v>8345.525501258526</v>
       </c>
       <c r="CE211" t="n">
-        <v>7184</v>
+        <v>8345.525501258526</v>
       </c>
       <c r="CF211" t="n">
-        <v>4.821476510067114</v>
+        <v>5.601023826348004</v>
       </c>
     </row>
     <row r="212">
@@ -68728,16 +68728,16 @@
         <v>485000</v>
       </c>
       <c r="CC212" t="n">
-        <v>414156.53</v>
+        <v>422434.3025730625</v>
       </c>
       <c r="CD212" t="n">
-        <v>70843.46999999997</v>
+        <v>62565.69742693746</v>
       </c>
       <c r="CE212" t="n">
-        <v>70843.46999999997</v>
+        <v>62565.69742693746</v>
       </c>
       <c r="CF212" t="n">
-        <v>14.60690103092783</v>
+        <v>12.90014379936855</v>
       </c>
     </row>
     <row r="213">
@@ -69056,16 +69056,16 @@
         <v>155000</v>
       </c>
       <c r="CC213" t="n">
-        <v>170298.35</v>
+        <v>172494.7612557134</v>
       </c>
       <c r="CD213" t="n">
-        <v>-15298.35000000001</v>
+        <v>-17494.76125571344</v>
       </c>
       <c r="CE213" t="n">
-        <v>15298.35000000001</v>
+        <v>17494.76125571344</v>
       </c>
       <c r="CF213" t="n">
-        <v>9.869903225806455</v>
+        <v>11.28694274562157</v>
       </c>
     </row>
     <row r="214">
@@ -69380,16 +69380,16 @@
         <v>202500</v>
       </c>
       <c r="CC214" t="n">
-        <v>193987.39</v>
+        <v>193414.5388617751</v>
       </c>
       <c r="CD214" t="n">
-        <v>8512.609999999986</v>
+        <v>9085.461138224928</v>
       </c>
       <c r="CE214" t="n">
-        <v>8512.609999999986</v>
+        <v>9085.461138224928</v>
       </c>
       <c r="CF214" t="n">
-        <v>4.203758024691351</v>
+        <v>4.486647475666631</v>
       </c>
     </row>
     <row r="215">
@@ -69704,16 +69704,16 @@
         <v>134000</v>
       </c>
       <c r="CC215" t="n">
-        <v>129391.5</v>
+        <v>130295.8912409448</v>
       </c>
       <c r="CD215" t="n">
-        <v>4608.5</v>
+        <v>3704.108759055234</v>
       </c>
       <c r="CE215" t="n">
-        <v>4608.5</v>
+        <v>3704.108759055234</v>
       </c>
       <c r="CF215" t="n">
-        <v>3.439179104477612</v>
+        <v>2.764260267951667</v>
       </c>
     </row>
     <row r="216">
@@ -70024,16 +70024,16 @@
         <v>156000</v>
       </c>
       <c r="CC216" t="n">
-        <v>145227.33</v>
+        <v>145503.4306910874</v>
       </c>
       <c r="CD216" t="n">
-        <v>10772.67000000001</v>
+        <v>10496.56930891259</v>
       </c>
       <c r="CE216" t="n">
-        <v>10772.67000000001</v>
+        <v>10496.56930891259</v>
       </c>
       <c r="CF216" t="n">
-        <v>6.905557692307701</v>
+        <v>6.728570069815759</v>
       </c>
     </row>
     <row r="217">
@@ -70342,16 +70342,16 @@
         <v>465000</v>
       </c>
       <c r="CC217" t="n">
-        <v>346128.53</v>
+        <v>362833.6896804388</v>
       </c>
       <c r="CD217" t="n">
-        <v>118871.47</v>
+        <v>102166.3103195612</v>
       </c>
       <c r="CE217" t="n">
-        <v>118871.47</v>
+        <v>102166.3103195612</v>
       </c>
       <c r="CF217" t="n">
-        <v>25.56375698924731</v>
+        <v>21.97124953108842</v>
       </c>
     </row>
     <row r="218">
@@ -70664,16 +70664,16 @@
         <v>250000</v>
       </c>
       <c r="CC218" t="n">
-        <v>201625.59</v>
+        <v>208390.7305205344</v>
       </c>
       <c r="CD218" t="n">
-        <v>48374.41</v>
+        <v>41609.26947946558</v>
       </c>
       <c r="CE218" t="n">
-        <v>48374.41</v>
+        <v>41609.26947946558</v>
       </c>
       <c r="CF218" t="n">
-        <v>19.349764</v>
+        <v>16.64370779178623</v>
       </c>
     </row>
     <row r="219">
@@ -70978,16 +70978,16 @@
         <v>205950</v>
       </c>
       <c r="CC219" t="n">
-        <v>191849.94</v>
+        <v>194206.1391606915</v>
       </c>
       <c r="CD219" t="n">
-        <v>14100.06</v>
+        <v>11743.8608393085</v>
       </c>
       <c r="CE219" t="n">
-        <v>14100.06</v>
+        <v>11743.8608393085</v>
       </c>
       <c r="CF219" t="n">
-        <v>6.846351056081572</v>
+        <v>5.702287370385289</v>
       </c>
     </row>
     <row r="220">
@@ -71302,16 +71302,16 @@
         <v>244000</v>
       </c>
       <c r="CC220" t="n">
-        <v>265139.8</v>
+        <v>263408.1339134833</v>
       </c>
       <c r="CD220" t="n">
-        <v>-21139.79999999999</v>
+        <v>-19408.1339134833</v>
       </c>
       <c r="CE220" t="n">
-        <v>21139.79999999999</v>
+        <v>19408.1339134833</v>
       </c>
       <c r="CF220" t="n">
-        <v>8.663852459016388</v>
+        <v>7.954153243230859</v>
       </c>
     </row>
   </sheetData>

</xml_diff>